<commit_message>
Restore bloomberg_prices.xlsx to pre-generated state
Excel files should not be modified directly — run
  python templates/create_bloomberg_template.py
to regenerate from the updated generator script.

https://claude.ai/code/session_016jjKeK1fziUHKc9iFqncks
</commit_message>
<xml_diff>
--- a/projects/02-pnl-dashboard/templates/bloomberg_prices.xlsx
+++ b/projects/02-pnl-dashboard/templates/bloomberg_prices.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Live MTM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Static" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="History" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +65,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +440,7 @@
   <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -444,7 +449,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BBG Ticker</t>
+          <t>CUSIP</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -465,701 +470,701 @@
     </row>
     <row r="2">
       <c r="B2">
-        <f>BDP(A2,"PX_LAST")</f>
+        <f>BDP(A2&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C2">
-        <f>BDP(A2,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A2&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>BDP(A2,"YLD_YTM_MID")</f>
+        <f>BDP(A2&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="B3">
-        <f>BDP(A3,"PX_LAST")</f>
+        <f>BDP(A3&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C3">
-        <f>BDP(A3,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A3&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>BDP(A3,"YLD_YTM_MID")</f>
+        <f>BDP(A3&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="B4">
-        <f>BDP(A4,"PX_LAST")</f>
+        <f>BDP(A4&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C4">
-        <f>BDP(A4,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A4&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>BDP(A4,"YLD_YTM_MID")</f>
+        <f>BDP(A4&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="B5">
-        <f>BDP(A5,"PX_LAST")</f>
+        <f>BDP(A5&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C5">
-        <f>BDP(A5,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A5&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>BDP(A5,"YLD_YTM_MID")</f>
+        <f>BDP(A5&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6">
-        <f>BDP(A6,"PX_LAST")</f>
+        <f>BDP(A6&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>BDP(A6,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A6&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>BDP(A6,"YLD_YTM_MID")</f>
+        <f>BDP(A6&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7">
-        <f>BDP(A7,"PX_LAST")</f>
+        <f>BDP(A7&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C7">
-        <f>BDP(A7,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A7&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D7">
-        <f>BDP(A7,"YLD_YTM_MID")</f>
+        <f>BDP(A7&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8">
-        <f>BDP(A8,"PX_LAST")</f>
+        <f>BDP(A8&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C8">
-        <f>BDP(A8,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A8&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D8">
-        <f>BDP(A8,"YLD_YTM_MID")</f>
+        <f>BDP(A8&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9">
-        <f>BDP(A9,"PX_LAST")</f>
+        <f>BDP(A9&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C9">
-        <f>BDP(A9,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A9&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D9">
-        <f>BDP(A9,"YLD_YTM_MID")</f>
+        <f>BDP(A9&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10">
-        <f>BDP(A10,"PX_LAST")</f>
+        <f>BDP(A10&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C10">
-        <f>BDP(A10,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A10&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D10">
-        <f>BDP(A10,"YLD_YTM_MID")</f>
+        <f>BDP(A10&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="B11">
-        <f>BDP(A11,"PX_LAST")</f>
+        <f>BDP(A11&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>BDP(A11,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A11&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D11">
-        <f>BDP(A11,"YLD_YTM_MID")</f>
+        <f>BDP(A11&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="B12">
-        <f>BDP(A12,"PX_LAST")</f>
+        <f>BDP(A12&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>BDP(A12,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A12&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>BDP(A12,"YLD_YTM_MID")</f>
+        <f>BDP(A12&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13">
-        <f>BDP(A13,"PX_LAST")</f>
+        <f>BDP(A13&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>BDP(A13,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A13&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D13">
-        <f>BDP(A13,"YLD_YTM_MID")</f>
+        <f>BDP(A13&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14">
-        <f>BDP(A14,"PX_LAST")</f>
+        <f>BDP(A14&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>BDP(A14,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A14&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D14">
-        <f>BDP(A14,"YLD_YTM_MID")</f>
+        <f>BDP(A14&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="B15">
-        <f>BDP(A15,"PX_LAST")</f>
+        <f>BDP(A15&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>BDP(A15,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A15&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D15">
-        <f>BDP(A15,"YLD_YTM_MID")</f>
+        <f>BDP(A15&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16">
-        <f>BDP(A16,"PX_LAST")</f>
+        <f>BDP(A16&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>BDP(A16,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A16&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D16">
-        <f>BDP(A16,"YLD_YTM_MID")</f>
+        <f>BDP(A16&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17">
-        <f>BDP(A17,"PX_LAST")</f>
+        <f>BDP(A17&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>BDP(A17,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A17&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D17">
-        <f>BDP(A17,"YLD_YTM_MID")</f>
+        <f>BDP(A17&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18">
-        <f>BDP(A18,"PX_LAST")</f>
+        <f>BDP(A18&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>BDP(A18,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A18&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D18">
-        <f>BDP(A18,"YLD_YTM_MID")</f>
+        <f>BDP(A18&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19">
-        <f>BDP(A19,"PX_LAST")</f>
+        <f>BDP(A19&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>BDP(A19,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A19&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D19">
-        <f>BDP(A19,"YLD_YTM_MID")</f>
+        <f>BDP(A19&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20">
-        <f>BDP(A20,"PX_LAST")</f>
+        <f>BDP(A20&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>BDP(A20,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A20&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D20">
-        <f>BDP(A20,"YLD_YTM_MID")</f>
+        <f>BDP(A20&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21">
-        <f>BDP(A21,"PX_LAST")</f>
+        <f>BDP(A21&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>BDP(A21,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A21&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D21">
-        <f>BDP(A21,"YLD_YTM_MID")</f>
+        <f>BDP(A21&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="B22">
-        <f>BDP(A22,"PX_LAST")</f>
+        <f>BDP(A22&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>BDP(A22,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A22&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D22">
-        <f>BDP(A22,"YLD_YTM_MID")</f>
+        <f>BDP(A22&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="B23">
-        <f>BDP(A23,"PX_LAST")</f>
+        <f>BDP(A23&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>BDP(A23,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A23&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>BDP(A23,"YLD_YTM_MID")</f>
+        <f>BDP(A23&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24">
-        <f>BDP(A24,"PX_LAST")</f>
+        <f>BDP(A24&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>BDP(A24,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A24&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>BDP(A24,"YLD_YTM_MID")</f>
+        <f>BDP(A24&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25">
-        <f>BDP(A25,"PX_LAST")</f>
+        <f>BDP(A25&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>BDP(A25,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A25&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>BDP(A25,"YLD_YTM_MID")</f>
+        <f>BDP(A25&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26">
-        <f>BDP(A26,"PX_LAST")</f>
+        <f>BDP(A26&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>BDP(A26,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A26&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D26">
-        <f>BDP(A26,"YLD_YTM_MID")</f>
+        <f>BDP(A26&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27">
-        <f>BDP(A27,"PX_LAST")</f>
+        <f>BDP(A27&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>BDP(A27,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A27&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>BDP(A27,"YLD_YTM_MID")</f>
+        <f>BDP(A27&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28">
-        <f>BDP(A28,"PX_LAST")</f>
+        <f>BDP(A28&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>BDP(A28,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A28&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D28">
-        <f>BDP(A28,"YLD_YTM_MID")</f>
+        <f>BDP(A28&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29">
-        <f>BDP(A29,"PX_LAST")</f>
+        <f>BDP(A29&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>BDP(A29,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A29&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D29">
-        <f>BDP(A29,"YLD_YTM_MID")</f>
+        <f>BDP(A29&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30">
-        <f>BDP(A30,"PX_LAST")</f>
+        <f>BDP(A30&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>BDP(A30,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A30&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D30">
-        <f>BDP(A30,"YLD_YTM_MID")</f>
+        <f>BDP(A30&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="B31">
-        <f>BDP(A31,"PX_LAST")</f>
+        <f>BDP(A31&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>BDP(A31,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A31&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D31">
-        <f>BDP(A31,"YLD_YTM_MID")</f>
+        <f>BDP(A31&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32">
-        <f>BDP(A32,"PX_LAST")</f>
+        <f>BDP(A32&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>BDP(A32,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A32&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D32">
-        <f>BDP(A32,"YLD_YTM_MID")</f>
+        <f>BDP(A32&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33">
-        <f>BDP(A33,"PX_LAST")</f>
+        <f>BDP(A33&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C33">
-        <f>BDP(A33,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A33&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>BDP(A33,"YLD_YTM_MID")</f>
+        <f>BDP(A33&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34">
-        <f>BDP(A34,"PX_LAST")</f>
+        <f>BDP(A34&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C34">
-        <f>BDP(A34,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A34&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>BDP(A34,"YLD_YTM_MID")</f>
+        <f>BDP(A34&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35">
-        <f>BDP(A35,"PX_LAST")</f>
+        <f>BDP(A35&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C35">
-        <f>BDP(A35,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A35&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D35">
-        <f>BDP(A35,"YLD_YTM_MID")</f>
+        <f>BDP(A35&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36">
-        <f>BDP(A36,"PX_LAST")</f>
+        <f>BDP(A36&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C36">
-        <f>BDP(A36,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A36&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D36">
-        <f>BDP(A36,"YLD_YTM_MID")</f>
+        <f>BDP(A36&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37">
-        <f>BDP(A37,"PX_LAST")</f>
+        <f>BDP(A37&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C37">
-        <f>BDP(A37,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A37&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D37">
-        <f>BDP(A37,"YLD_YTM_MID")</f>
+        <f>BDP(A37&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="B38">
-        <f>BDP(A38,"PX_LAST")</f>
+        <f>BDP(A38&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C38">
-        <f>BDP(A38,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A38&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D38">
-        <f>BDP(A38,"YLD_YTM_MID")</f>
+        <f>BDP(A38&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39">
-        <f>BDP(A39,"PX_LAST")</f>
+        <f>BDP(A39&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C39">
-        <f>BDP(A39,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A39&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D39">
-        <f>BDP(A39,"YLD_YTM_MID")</f>
+        <f>BDP(A39&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="B40">
-        <f>BDP(A40,"PX_LAST")</f>
+        <f>BDP(A40&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C40">
-        <f>BDP(A40,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A40&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D40">
-        <f>BDP(A40,"YLD_YTM_MID")</f>
+        <f>BDP(A40&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="B41">
-        <f>BDP(A41,"PX_LAST")</f>
+        <f>BDP(A41&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C41">
-        <f>BDP(A41,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A41&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D41">
-        <f>BDP(A41,"YLD_YTM_MID")</f>
+        <f>BDP(A41&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42">
-        <f>BDP(A42,"PX_LAST")</f>
+        <f>BDP(A42&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C42">
-        <f>BDP(A42,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A42&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D42">
-        <f>BDP(A42,"YLD_YTM_MID")</f>
+        <f>BDP(A42&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43">
-        <f>BDP(A43,"PX_LAST")</f>
+        <f>BDP(A43&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C43">
-        <f>BDP(A43,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A43&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D43">
-        <f>BDP(A43,"YLD_YTM_MID")</f>
+        <f>BDP(A43&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44">
-        <f>BDP(A44,"PX_LAST")</f>
+        <f>BDP(A44&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C44">
-        <f>BDP(A44,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A44&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D44">
-        <f>BDP(A44,"YLD_YTM_MID")</f>
+        <f>BDP(A44&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45">
-        <f>BDP(A45,"PX_LAST")</f>
+        <f>BDP(A45&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C45">
-        <f>BDP(A45,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A45&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D45">
-        <f>BDP(A45,"YLD_YTM_MID")</f>
+        <f>BDP(A45&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="B46">
-        <f>BDP(A46,"PX_LAST")</f>
+        <f>BDP(A46&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C46">
-        <f>BDP(A46,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A46&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D46">
-        <f>BDP(A46,"YLD_YTM_MID")</f>
+        <f>BDP(A46&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47">
-        <f>BDP(A47,"PX_LAST")</f>
+        <f>BDP(A47&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C47">
-        <f>BDP(A47,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A47&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D47">
-        <f>BDP(A47,"YLD_YTM_MID")</f>
+        <f>BDP(A47&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="B48">
-        <f>BDP(A48,"PX_LAST")</f>
+        <f>BDP(A48&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C48">
-        <f>BDP(A48,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A48&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D48">
-        <f>BDP(A48,"YLD_YTM_MID")</f>
+        <f>BDP(A48&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="B49">
-        <f>BDP(A49,"PX_LAST")</f>
+        <f>BDP(A49&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C49">
-        <f>BDP(A49,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A49&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D49">
-        <f>BDP(A49,"YLD_YTM_MID")</f>
+        <f>BDP(A49&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="B50">
-        <f>BDP(A50,"PX_LAST")</f>
+        <f>BDP(A50&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C50">
-        <f>BDP(A50,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A50&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D50">
-        <f>BDP(A50,"YLD_YTM_MID")</f>
+        <f>BDP(A50&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="B51">
-        <f>BDP(A51,"PX_LAST")</f>
+        <f>BDP(A51&amp;" Corp","PX_LAST")</f>
         <v/>
       </c>
       <c r="C51">
-        <f>BDP(A51,"YAS_ASW_SPREAD")</f>
+        <f>BDP(A51&amp;" Corp","YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D51">
-        <f>BDP(A51,"YLD_YTM_MID")</f>
+        <f>BDP(A51&amp;" Corp","YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
@@ -1177,7 +1182,7 @@
   <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -1191,7 +1196,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>bbg_ticker</t>
+          <t>cusip</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1237,1701 +1242,1701 @@
     </row>
     <row r="2">
       <c r="B2">
-        <f>BDP(A2,"SECURITY_DES")</f>
+        <f>BDP(A2&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C2">
-        <f>BDP(A2,"CRNCY")</f>
+        <f>BDP(A2&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>BDP(A2,"CNTRY_OF_RISK")</f>
+        <f>BDP(A2&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E2">
-        <f>BDP(A2,"CPN")/100</f>
+        <f>BDP(A2&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F2">
-        <f>BDP(A2,"CPN_FREQ")</f>
+        <f>BDP(A2&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G2">
-        <f>BDP(A2,"DAY_CNT_DES")</f>
+        <f>BDP(A2&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H2">
-        <f>BDP(A2,"MATURITY")</f>
+        <f>BDP(A2&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I2">
-        <f>BDP(A2,"FIRST_CPN_DT")</f>
+        <f>BDP(A2&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="B3">
-        <f>BDP(A3,"SECURITY_DES")</f>
+        <f>BDP(A3&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C3">
-        <f>BDP(A3,"CRNCY")</f>
+        <f>BDP(A3&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>BDP(A3,"CNTRY_OF_RISK")</f>
+        <f>BDP(A3&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E3">
-        <f>BDP(A3,"CPN")/100</f>
+        <f>BDP(A3&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F3">
-        <f>BDP(A3,"CPN_FREQ")</f>
+        <f>BDP(A3&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G3">
-        <f>BDP(A3,"DAY_CNT_DES")</f>
+        <f>BDP(A3&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H3">
-        <f>BDP(A3,"MATURITY")</f>
+        <f>BDP(A3&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I3">
-        <f>BDP(A3,"FIRST_CPN_DT")</f>
+        <f>BDP(A3&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="B4">
-        <f>BDP(A4,"SECURITY_DES")</f>
+        <f>BDP(A4&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C4">
-        <f>BDP(A4,"CRNCY")</f>
+        <f>BDP(A4&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>BDP(A4,"CNTRY_OF_RISK")</f>
+        <f>BDP(A4&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E4">
-        <f>BDP(A4,"CPN")/100</f>
+        <f>BDP(A4&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F4">
-        <f>BDP(A4,"CPN_FREQ")</f>
+        <f>BDP(A4&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G4">
-        <f>BDP(A4,"DAY_CNT_DES")</f>
+        <f>BDP(A4&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H4">
-        <f>BDP(A4,"MATURITY")</f>
+        <f>BDP(A4&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I4">
-        <f>BDP(A4,"FIRST_CPN_DT")</f>
+        <f>BDP(A4&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="B5">
-        <f>BDP(A5,"SECURITY_DES")</f>
+        <f>BDP(A5&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C5">
-        <f>BDP(A5,"CRNCY")</f>
+        <f>BDP(A5&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>BDP(A5,"CNTRY_OF_RISK")</f>
+        <f>BDP(A5&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E5">
-        <f>BDP(A5,"CPN")/100</f>
+        <f>BDP(A5&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F5">
-        <f>BDP(A5,"CPN_FREQ")</f>
+        <f>BDP(A5&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G5">
-        <f>BDP(A5,"DAY_CNT_DES")</f>
+        <f>BDP(A5&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H5">
-        <f>BDP(A5,"MATURITY")</f>
+        <f>BDP(A5&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I5">
-        <f>BDP(A5,"FIRST_CPN_DT")</f>
+        <f>BDP(A5&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6">
-        <f>BDP(A6,"SECURITY_DES")</f>
+        <f>BDP(A6&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>BDP(A6,"CRNCY")</f>
+        <f>BDP(A6&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>BDP(A6,"CNTRY_OF_RISK")</f>
+        <f>BDP(A6&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E6">
-        <f>BDP(A6,"CPN")/100</f>
+        <f>BDP(A6&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F6">
-        <f>BDP(A6,"CPN_FREQ")</f>
+        <f>BDP(A6&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G6">
-        <f>BDP(A6,"DAY_CNT_DES")</f>
+        <f>BDP(A6&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H6">
-        <f>BDP(A6,"MATURITY")</f>
+        <f>BDP(A6&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I6">
-        <f>BDP(A6,"FIRST_CPN_DT")</f>
+        <f>BDP(A6&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7">
-        <f>BDP(A7,"SECURITY_DES")</f>
+        <f>BDP(A7&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C7">
-        <f>BDP(A7,"CRNCY")</f>
+        <f>BDP(A7&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D7">
-        <f>BDP(A7,"CNTRY_OF_RISK")</f>
+        <f>BDP(A7&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E7">
-        <f>BDP(A7,"CPN")/100</f>
+        <f>BDP(A7&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F7">
-        <f>BDP(A7,"CPN_FREQ")</f>
+        <f>BDP(A7&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G7">
-        <f>BDP(A7,"DAY_CNT_DES")</f>
+        <f>BDP(A7&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H7">
-        <f>BDP(A7,"MATURITY")</f>
+        <f>BDP(A7&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I7">
-        <f>BDP(A7,"FIRST_CPN_DT")</f>
+        <f>BDP(A7&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8">
-        <f>BDP(A8,"SECURITY_DES")</f>
+        <f>BDP(A8&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C8">
-        <f>BDP(A8,"CRNCY")</f>
+        <f>BDP(A8&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D8">
-        <f>BDP(A8,"CNTRY_OF_RISK")</f>
+        <f>BDP(A8&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E8">
-        <f>BDP(A8,"CPN")/100</f>
+        <f>BDP(A8&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F8">
-        <f>BDP(A8,"CPN_FREQ")</f>
+        <f>BDP(A8&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G8">
-        <f>BDP(A8,"DAY_CNT_DES")</f>
+        <f>BDP(A8&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H8">
-        <f>BDP(A8,"MATURITY")</f>
+        <f>BDP(A8&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I8">
-        <f>BDP(A8,"FIRST_CPN_DT")</f>
+        <f>BDP(A8&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9">
-        <f>BDP(A9,"SECURITY_DES")</f>
+        <f>BDP(A9&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C9">
-        <f>BDP(A9,"CRNCY")</f>
+        <f>BDP(A9&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D9">
-        <f>BDP(A9,"CNTRY_OF_RISK")</f>
+        <f>BDP(A9&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E9">
-        <f>BDP(A9,"CPN")/100</f>
+        <f>BDP(A9&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F9">
-        <f>BDP(A9,"CPN_FREQ")</f>
+        <f>BDP(A9&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G9">
-        <f>BDP(A9,"DAY_CNT_DES")</f>
+        <f>BDP(A9&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H9">
-        <f>BDP(A9,"MATURITY")</f>
+        <f>BDP(A9&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I9">
-        <f>BDP(A9,"FIRST_CPN_DT")</f>
+        <f>BDP(A9&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10">
-        <f>BDP(A10,"SECURITY_DES")</f>
+        <f>BDP(A10&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C10">
-        <f>BDP(A10,"CRNCY")</f>
+        <f>BDP(A10&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D10">
-        <f>BDP(A10,"CNTRY_OF_RISK")</f>
+        <f>BDP(A10&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E10">
-        <f>BDP(A10,"CPN")/100</f>
+        <f>BDP(A10&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F10">
-        <f>BDP(A10,"CPN_FREQ")</f>
+        <f>BDP(A10&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G10">
-        <f>BDP(A10,"DAY_CNT_DES")</f>
+        <f>BDP(A10&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H10">
-        <f>BDP(A10,"MATURITY")</f>
+        <f>BDP(A10&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I10">
-        <f>BDP(A10,"FIRST_CPN_DT")</f>
+        <f>BDP(A10&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="B11">
-        <f>BDP(A11,"SECURITY_DES")</f>
+        <f>BDP(A11&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>BDP(A11,"CRNCY")</f>
+        <f>BDP(A11&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D11">
-        <f>BDP(A11,"CNTRY_OF_RISK")</f>
+        <f>BDP(A11&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E11">
-        <f>BDP(A11,"CPN")/100</f>
+        <f>BDP(A11&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F11">
-        <f>BDP(A11,"CPN_FREQ")</f>
+        <f>BDP(A11&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G11">
-        <f>BDP(A11,"DAY_CNT_DES")</f>
+        <f>BDP(A11&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H11">
-        <f>BDP(A11,"MATURITY")</f>
+        <f>BDP(A11&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I11">
-        <f>BDP(A11,"FIRST_CPN_DT")</f>
+        <f>BDP(A11&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="B12">
-        <f>BDP(A12,"SECURITY_DES")</f>
+        <f>BDP(A12&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>BDP(A12,"CRNCY")</f>
+        <f>BDP(A12&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>BDP(A12,"CNTRY_OF_RISK")</f>
+        <f>BDP(A12&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E12">
-        <f>BDP(A12,"CPN")/100</f>
+        <f>BDP(A12&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F12">
-        <f>BDP(A12,"CPN_FREQ")</f>
+        <f>BDP(A12&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G12">
-        <f>BDP(A12,"DAY_CNT_DES")</f>
+        <f>BDP(A12&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H12">
-        <f>BDP(A12,"MATURITY")</f>
+        <f>BDP(A12&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I12">
-        <f>BDP(A12,"FIRST_CPN_DT")</f>
+        <f>BDP(A12&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13">
-        <f>BDP(A13,"SECURITY_DES")</f>
+        <f>BDP(A13&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>BDP(A13,"CRNCY")</f>
+        <f>BDP(A13&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D13">
-        <f>BDP(A13,"CNTRY_OF_RISK")</f>
+        <f>BDP(A13&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E13">
-        <f>BDP(A13,"CPN")/100</f>
+        <f>BDP(A13&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F13">
-        <f>BDP(A13,"CPN_FREQ")</f>
+        <f>BDP(A13&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G13">
-        <f>BDP(A13,"DAY_CNT_DES")</f>
+        <f>BDP(A13&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H13">
-        <f>BDP(A13,"MATURITY")</f>
+        <f>BDP(A13&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I13">
-        <f>BDP(A13,"FIRST_CPN_DT")</f>
+        <f>BDP(A13&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14">
-        <f>BDP(A14,"SECURITY_DES")</f>
+        <f>BDP(A14&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>BDP(A14,"CRNCY")</f>
+        <f>BDP(A14&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D14">
-        <f>BDP(A14,"CNTRY_OF_RISK")</f>
+        <f>BDP(A14&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E14">
-        <f>BDP(A14,"CPN")/100</f>
+        <f>BDP(A14&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F14">
-        <f>BDP(A14,"CPN_FREQ")</f>
+        <f>BDP(A14&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G14">
-        <f>BDP(A14,"DAY_CNT_DES")</f>
+        <f>BDP(A14&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H14">
-        <f>BDP(A14,"MATURITY")</f>
+        <f>BDP(A14&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I14">
-        <f>BDP(A14,"FIRST_CPN_DT")</f>
+        <f>BDP(A14&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="B15">
-        <f>BDP(A15,"SECURITY_DES")</f>
+        <f>BDP(A15&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>BDP(A15,"CRNCY")</f>
+        <f>BDP(A15&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D15">
-        <f>BDP(A15,"CNTRY_OF_RISK")</f>
+        <f>BDP(A15&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E15">
-        <f>BDP(A15,"CPN")/100</f>
+        <f>BDP(A15&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F15">
-        <f>BDP(A15,"CPN_FREQ")</f>
+        <f>BDP(A15&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G15">
-        <f>BDP(A15,"DAY_CNT_DES")</f>
+        <f>BDP(A15&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H15">
-        <f>BDP(A15,"MATURITY")</f>
+        <f>BDP(A15&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I15">
-        <f>BDP(A15,"FIRST_CPN_DT")</f>
+        <f>BDP(A15&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16">
-        <f>BDP(A16,"SECURITY_DES")</f>
+        <f>BDP(A16&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>BDP(A16,"CRNCY")</f>
+        <f>BDP(A16&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D16">
-        <f>BDP(A16,"CNTRY_OF_RISK")</f>
+        <f>BDP(A16&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E16">
-        <f>BDP(A16,"CPN")/100</f>
+        <f>BDP(A16&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F16">
-        <f>BDP(A16,"CPN_FREQ")</f>
+        <f>BDP(A16&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G16">
-        <f>BDP(A16,"DAY_CNT_DES")</f>
+        <f>BDP(A16&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H16">
-        <f>BDP(A16,"MATURITY")</f>
+        <f>BDP(A16&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I16">
-        <f>BDP(A16,"FIRST_CPN_DT")</f>
+        <f>BDP(A16&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17">
-        <f>BDP(A17,"SECURITY_DES")</f>
+        <f>BDP(A17&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>BDP(A17,"CRNCY")</f>
+        <f>BDP(A17&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D17">
-        <f>BDP(A17,"CNTRY_OF_RISK")</f>
+        <f>BDP(A17&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E17">
-        <f>BDP(A17,"CPN")/100</f>
+        <f>BDP(A17&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F17">
-        <f>BDP(A17,"CPN_FREQ")</f>
+        <f>BDP(A17&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G17">
-        <f>BDP(A17,"DAY_CNT_DES")</f>
+        <f>BDP(A17&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H17">
-        <f>BDP(A17,"MATURITY")</f>
+        <f>BDP(A17&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I17">
-        <f>BDP(A17,"FIRST_CPN_DT")</f>
+        <f>BDP(A17&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18">
-        <f>BDP(A18,"SECURITY_DES")</f>
+        <f>BDP(A18&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>BDP(A18,"CRNCY")</f>
+        <f>BDP(A18&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D18">
-        <f>BDP(A18,"CNTRY_OF_RISK")</f>
+        <f>BDP(A18&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E18">
-        <f>BDP(A18,"CPN")/100</f>
+        <f>BDP(A18&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F18">
-        <f>BDP(A18,"CPN_FREQ")</f>
+        <f>BDP(A18&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G18">
-        <f>BDP(A18,"DAY_CNT_DES")</f>
+        <f>BDP(A18&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H18">
-        <f>BDP(A18,"MATURITY")</f>
+        <f>BDP(A18&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I18">
-        <f>BDP(A18,"FIRST_CPN_DT")</f>
+        <f>BDP(A18&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19">
-        <f>BDP(A19,"SECURITY_DES")</f>
+        <f>BDP(A19&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>BDP(A19,"CRNCY")</f>
+        <f>BDP(A19&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D19">
-        <f>BDP(A19,"CNTRY_OF_RISK")</f>
+        <f>BDP(A19&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E19">
-        <f>BDP(A19,"CPN")/100</f>
+        <f>BDP(A19&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F19">
-        <f>BDP(A19,"CPN_FREQ")</f>
+        <f>BDP(A19&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G19">
-        <f>BDP(A19,"DAY_CNT_DES")</f>
+        <f>BDP(A19&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H19">
-        <f>BDP(A19,"MATURITY")</f>
+        <f>BDP(A19&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I19">
-        <f>BDP(A19,"FIRST_CPN_DT")</f>
+        <f>BDP(A19&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20">
-        <f>BDP(A20,"SECURITY_DES")</f>
+        <f>BDP(A20&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>BDP(A20,"CRNCY")</f>
+        <f>BDP(A20&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D20">
-        <f>BDP(A20,"CNTRY_OF_RISK")</f>
+        <f>BDP(A20&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E20">
-        <f>BDP(A20,"CPN")/100</f>
+        <f>BDP(A20&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F20">
-        <f>BDP(A20,"CPN_FREQ")</f>
+        <f>BDP(A20&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G20">
-        <f>BDP(A20,"DAY_CNT_DES")</f>
+        <f>BDP(A20&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H20">
-        <f>BDP(A20,"MATURITY")</f>
+        <f>BDP(A20&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I20">
-        <f>BDP(A20,"FIRST_CPN_DT")</f>
+        <f>BDP(A20&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21">
-        <f>BDP(A21,"SECURITY_DES")</f>
+        <f>BDP(A21&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>BDP(A21,"CRNCY")</f>
+        <f>BDP(A21&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D21">
-        <f>BDP(A21,"CNTRY_OF_RISK")</f>
+        <f>BDP(A21&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E21">
-        <f>BDP(A21,"CPN")/100</f>
+        <f>BDP(A21&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F21">
-        <f>BDP(A21,"CPN_FREQ")</f>
+        <f>BDP(A21&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G21">
-        <f>BDP(A21,"DAY_CNT_DES")</f>
+        <f>BDP(A21&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H21">
-        <f>BDP(A21,"MATURITY")</f>
+        <f>BDP(A21&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I21">
-        <f>BDP(A21,"FIRST_CPN_DT")</f>
+        <f>BDP(A21&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="B22">
-        <f>BDP(A22,"SECURITY_DES")</f>
+        <f>BDP(A22&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>BDP(A22,"CRNCY")</f>
+        <f>BDP(A22&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D22">
-        <f>BDP(A22,"CNTRY_OF_RISK")</f>
+        <f>BDP(A22&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E22">
-        <f>BDP(A22,"CPN")/100</f>
+        <f>BDP(A22&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F22">
-        <f>BDP(A22,"CPN_FREQ")</f>
+        <f>BDP(A22&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G22">
-        <f>BDP(A22,"DAY_CNT_DES")</f>
+        <f>BDP(A22&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H22">
-        <f>BDP(A22,"MATURITY")</f>
+        <f>BDP(A22&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I22">
-        <f>BDP(A22,"FIRST_CPN_DT")</f>
+        <f>BDP(A22&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="B23">
-        <f>BDP(A23,"SECURITY_DES")</f>
+        <f>BDP(A23&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>BDP(A23,"CRNCY")</f>
+        <f>BDP(A23&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>BDP(A23,"CNTRY_OF_RISK")</f>
+        <f>BDP(A23&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E23">
-        <f>BDP(A23,"CPN")/100</f>
+        <f>BDP(A23&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F23">
-        <f>BDP(A23,"CPN_FREQ")</f>
+        <f>BDP(A23&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G23">
-        <f>BDP(A23,"DAY_CNT_DES")</f>
+        <f>BDP(A23&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H23">
-        <f>BDP(A23,"MATURITY")</f>
+        <f>BDP(A23&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I23">
-        <f>BDP(A23,"FIRST_CPN_DT")</f>
+        <f>BDP(A23&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24">
-        <f>BDP(A24,"SECURITY_DES")</f>
+        <f>BDP(A24&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>BDP(A24,"CRNCY")</f>
+        <f>BDP(A24&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>BDP(A24,"CNTRY_OF_RISK")</f>
+        <f>BDP(A24&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E24">
-        <f>BDP(A24,"CPN")/100</f>
+        <f>BDP(A24&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F24">
-        <f>BDP(A24,"CPN_FREQ")</f>
+        <f>BDP(A24&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G24">
-        <f>BDP(A24,"DAY_CNT_DES")</f>
+        <f>BDP(A24&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H24">
-        <f>BDP(A24,"MATURITY")</f>
+        <f>BDP(A24&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I24">
-        <f>BDP(A24,"FIRST_CPN_DT")</f>
+        <f>BDP(A24&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25">
-        <f>BDP(A25,"SECURITY_DES")</f>
+        <f>BDP(A25&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>BDP(A25,"CRNCY")</f>
+        <f>BDP(A25&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>BDP(A25,"CNTRY_OF_RISK")</f>
+        <f>BDP(A25&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E25">
-        <f>BDP(A25,"CPN")/100</f>
+        <f>BDP(A25&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F25">
-        <f>BDP(A25,"CPN_FREQ")</f>
+        <f>BDP(A25&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G25">
-        <f>BDP(A25,"DAY_CNT_DES")</f>
+        <f>BDP(A25&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H25">
-        <f>BDP(A25,"MATURITY")</f>
+        <f>BDP(A25&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I25">
-        <f>BDP(A25,"FIRST_CPN_DT")</f>
+        <f>BDP(A25&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26">
-        <f>BDP(A26,"SECURITY_DES")</f>
+        <f>BDP(A26&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>BDP(A26,"CRNCY")</f>
+        <f>BDP(A26&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D26">
-        <f>BDP(A26,"CNTRY_OF_RISK")</f>
+        <f>BDP(A26&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E26">
-        <f>BDP(A26,"CPN")/100</f>
+        <f>BDP(A26&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F26">
-        <f>BDP(A26,"CPN_FREQ")</f>
+        <f>BDP(A26&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G26">
-        <f>BDP(A26,"DAY_CNT_DES")</f>
+        <f>BDP(A26&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H26">
-        <f>BDP(A26,"MATURITY")</f>
+        <f>BDP(A26&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I26">
-        <f>BDP(A26,"FIRST_CPN_DT")</f>
+        <f>BDP(A26&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27">
-        <f>BDP(A27,"SECURITY_DES")</f>
+        <f>BDP(A27&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>BDP(A27,"CRNCY")</f>
+        <f>BDP(A27&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>BDP(A27,"CNTRY_OF_RISK")</f>
+        <f>BDP(A27&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E27">
-        <f>BDP(A27,"CPN")/100</f>
+        <f>BDP(A27&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F27">
-        <f>BDP(A27,"CPN_FREQ")</f>
+        <f>BDP(A27&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G27">
-        <f>BDP(A27,"DAY_CNT_DES")</f>
+        <f>BDP(A27&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H27">
-        <f>BDP(A27,"MATURITY")</f>
+        <f>BDP(A27&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I27">
-        <f>BDP(A27,"FIRST_CPN_DT")</f>
+        <f>BDP(A27&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28">
-        <f>BDP(A28,"SECURITY_DES")</f>
+        <f>BDP(A28&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>BDP(A28,"CRNCY")</f>
+        <f>BDP(A28&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D28">
-        <f>BDP(A28,"CNTRY_OF_RISK")</f>
+        <f>BDP(A28&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E28">
-        <f>BDP(A28,"CPN")/100</f>
+        <f>BDP(A28&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F28">
-        <f>BDP(A28,"CPN_FREQ")</f>
+        <f>BDP(A28&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G28">
-        <f>BDP(A28,"DAY_CNT_DES")</f>
+        <f>BDP(A28&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H28">
-        <f>BDP(A28,"MATURITY")</f>
+        <f>BDP(A28&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I28">
-        <f>BDP(A28,"FIRST_CPN_DT")</f>
+        <f>BDP(A28&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29">
-        <f>BDP(A29,"SECURITY_DES")</f>
+        <f>BDP(A29&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>BDP(A29,"CRNCY")</f>
+        <f>BDP(A29&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D29">
-        <f>BDP(A29,"CNTRY_OF_RISK")</f>
+        <f>BDP(A29&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E29">
-        <f>BDP(A29,"CPN")/100</f>
+        <f>BDP(A29&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F29">
-        <f>BDP(A29,"CPN_FREQ")</f>
+        <f>BDP(A29&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G29">
-        <f>BDP(A29,"DAY_CNT_DES")</f>
+        <f>BDP(A29&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H29">
-        <f>BDP(A29,"MATURITY")</f>
+        <f>BDP(A29&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I29">
-        <f>BDP(A29,"FIRST_CPN_DT")</f>
+        <f>BDP(A29&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30">
-        <f>BDP(A30,"SECURITY_DES")</f>
+        <f>BDP(A30&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>BDP(A30,"CRNCY")</f>
+        <f>BDP(A30&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D30">
-        <f>BDP(A30,"CNTRY_OF_RISK")</f>
+        <f>BDP(A30&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E30">
-        <f>BDP(A30,"CPN")/100</f>
+        <f>BDP(A30&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F30">
-        <f>BDP(A30,"CPN_FREQ")</f>
+        <f>BDP(A30&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G30">
-        <f>BDP(A30,"DAY_CNT_DES")</f>
+        <f>BDP(A30&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H30">
-        <f>BDP(A30,"MATURITY")</f>
+        <f>BDP(A30&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I30">
-        <f>BDP(A30,"FIRST_CPN_DT")</f>
+        <f>BDP(A30&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="B31">
-        <f>BDP(A31,"SECURITY_DES")</f>
+        <f>BDP(A31&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>BDP(A31,"CRNCY")</f>
+        <f>BDP(A31&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D31">
-        <f>BDP(A31,"CNTRY_OF_RISK")</f>
+        <f>BDP(A31&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E31">
-        <f>BDP(A31,"CPN")/100</f>
+        <f>BDP(A31&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F31">
-        <f>BDP(A31,"CPN_FREQ")</f>
+        <f>BDP(A31&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G31">
-        <f>BDP(A31,"DAY_CNT_DES")</f>
+        <f>BDP(A31&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H31">
-        <f>BDP(A31,"MATURITY")</f>
+        <f>BDP(A31&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I31">
-        <f>BDP(A31,"FIRST_CPN_DT")</f>
+        <f>BDP(A31&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32">
-        <f>BDP(A32,"SECURITY_DES")</f>
+        <f>BDP(A32&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>BDP(A32,"CRNCY")</f>
+        <f>BDP(A32&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D32">
-        <f>BDP(A32,"CNTRY_OF_RISK")</f>
+        <f>BDP(A32&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E32">
-        <f>BDP(A32,"CPN")/100</f>
+        <f>BDP(A32&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F32">
-        <f>BDP(A32,"CPN_FREQ")</f>
+        <f>BDP(A32&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G32">
-        <f>BDP(A32,"DAY_CNT_DES")</f>
+        <f>BDP(A32&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H32">
-        <f>BDP(A32,"MATURITY")</f>
+        <f>BDP(A32&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I32">
-        <f>BDP(A32,"FIRST_CPN_DT")</f>
+        <f>BDP(A32&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33">
-        <f>BDP(A33,"SECURITY_DES")</f>
+        <f>BDP(A33&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C33">
-        <f>BDP(A33,"CRNCY")</f>
+        <f>BDP(A33&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>BDP(A33,"CNTRY_OF_RISK")</f>
+        <f>BDP(A33&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E33">
-        <f>BDP(A33,"CPN")/100</f>
+        <f>BDP(A33&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F33">
-        <f>BDP(A33,"CPN_FREQ")</f>
+        <f>BDP(A33&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G33">
-        <f>BDP(A33,"DAY_CNT_DES")</f>
+        <f>BDP(A33&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H33">
-        <f>BDP(A33,"MATURITY")</f>
+        <f>BDP(A33&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I33">
-        <f>BDP(A33,"FIRST_CPN_DT")</f>
+        <f>BDP(A33&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34">
-        <f>BDP(A34,"SECURITY_DES")</f>
+        <f>BDP(A34&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C34">
-        <f>BDP(A34,"CRNCY")</f>
+        <f>BDP(A34&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>BDP(A34,"CNTRY_OF_RISK")</f>
+        <f>BDP(A34&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E34">
-        <f>BDP(A34,"CPN")/100</f>
+        <f>BDP(A34&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F34">
-        <f>BDP(A34,"CPN_FREQ")</f>
+        <f>BDP(A34&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G34">
-        <f>BDP(A34,"DAY_CNT_DES")</f>
+        <f>BDP(A34&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H34">
-        <f>BDP(A34,"MATURITY")</f>
+        <f>BDP(A34&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I34">
-        <f>BDP(A34,"FIRST_CPN_DT")</f>
+        <f>BDP(A34&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35">
-        <f>BDP(A35,"SECURITY_DES")</f>
+        <f>BDP(A35&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C35">
-        <f>BDP(A35,"CRNCY")</f>
+        <f>BDP(A35&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D35">
-        <f>BDP(A35,"CNTRY_OF_RISK")</f>
+        <f>BDP(A35&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E35">
-        <f>BDP(A35,"CPN")/100</f>
+        <f>BDP(A35&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F35">
-        <f>BDP(A35,"CPN_FREQ")</f>
+        <f>BDP(A35&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G35">
-        <f>BDP(A35,"DAY_CNT_DES")</f>
+        <f>BDP(A35&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H35">
-        <f>BDP(A35,"MATURITY")</f>
+        <f>BDP(A35&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I35">
-        <f>BDP(A35,"FIRST_CPN_DT")</f>
+        <f>BDP(A35&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36">
-        <f>BDP(A36,"SECURITY_DES")</f>
+        <f>BDP(A36&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C36">
-        <f>BDP(A36,"CRNCY")</f>
+        <f>BDP(A36&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D36">
-        <f>BDP(A36,"CNTRY_OF_RISK")</f>
+        <f>BDP(A36&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E36">
-        <f>BDP(A36,"CPN")/100</f>
+        <f>BDP(A36&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F36">
-        <f>BDP(A36,"CPN_FREQ")</f>
+        <f>BDP(A36&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G36">
-        <f>BDP(A36,"DAY_CNT_DES")</f>
+        <f>BDP(A36&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H36">
-        <f>BDP(A36,"MATURITY")</f>
+        <f>BDP(A36&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I36">
-        <f>BDP(A36,"FIRST_CPN_DT")</f>
+        <f>BDP(A36&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37">
-        <f>BDP(A37,"SECURITY_DES")</f>
+        <f>BDP(A37&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C37">
-        <f>BDP(A37,"CRNCY")</f>
+        <f>BDP(A37&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D37">
-        <f>BDP(A37,"CNTRY_OF_RISK")</f>
+        <f>BDP(A37&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E37">
-        <f>BDP(A37,"CPN")/100</f>
+        <f>BDP(A37&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F37">
-        <f>BDP(A37,"CPN_FREQ")</f>
+        <f>BDP(A37&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G37">
-        <f>BDP(A37,"DAY_CNT_DES")</f>
+        <f>BDP(A37&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H37">
-        <f>BDP(A37,"MATURITY")</f>
+        <f>BDP(A37&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I37">
-        <f>BDP(A37,"FIRST_CPN_DT")</f>
+        <f>BDP(A37&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="B38">
-        <f>BDP(A38,"SECURITY_DES")</f>
+        <f>BDP(A38&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C38">
-        <f>BDP(A38,"CRNCY")</f>
+        <f>BDP(A38&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D38">
-        <f>BDP(A38,"CNTRY_OF_RISK")</f>
+        <f>BDP(A38&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E38">
-        <f>BDP(A38,"CPN")/100</f>
+        <f>BDP(A38&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F38">
-        <f>BDP(A38,"CPN_FREQ")</f>
+        <f>BDP(A38&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G38">
-        <f>BDP(A38,"DAY_CNT_DES")</f>
+        <f>BDP(A38&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H38">
-        <f>BDP(A38,"MATURITY")</f>
+        <f>BDP(A38&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I38">
-        <f>BDP(A38,"FIRST_CPN_DT")</f>
+        <f>BDP(A38&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39">
-        <f>BDP(A39,"SECURITY_DES")</f>
+        <f>BDP(A39&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C39">
-        <f>BDP(A39,"CRNCY")</f>
+        <f>BDP(A39&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D39">
-        <f>BDP(A39,"CNTRY_OF_RISK")</f>
+        <f>BDP(A39&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E39">
-        <f>BDP(A39,"CPN")/100</f>
+        <f>BDP(A39&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F39">
-        <f>BDP(A39,"CPN_FREQ")</f>
+        <f>BDP(A39&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G39">
-        <f>BDP(A39,"DAY_CNT_DES")</f>
+        <f>BDP(A39&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H39">
-        <f>BDP(A39,"MATURITY")</f>
+        <f>BDP(A39&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I39">
-        <f>BDP(A39,"FIRST_CPN_DT")</f>
+        <f>BDP(A39&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="B40">
-        <f>BDP(A40,"SECURITY_DES")</f>
+        <f>BDP(A40&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C40">
-        <f>BDP(A40,"CRNCY")</f>
+        <f>BDP(A40&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D40">
-        <f>BDP(A40,"CNTRY_OF_RISK")</f>
+        <f>BDP(A40&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E40">
-        <f>BDP(A40,"CPN")/100</f>
+        <f>BDP(A40&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F40">
-        <f>BDP(A40,"CPN_FREQ")</f>
+        <f>BDP(A40&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G40">
-        <f>BDP(A40,"DAY_CNT_DES")</f>
+        <f>BDP(A40&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H40">
-        <f>BDP(A40,"MATURITY")</f>
+        <f>BDP(A40&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I40">
-        <f>BDP(A40,"FIRST_CPN_DT")</f>
+        <f>BDP(A40&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="B41">
-        <f>BDP(A41,"SECURITY_DES")</f>
+        <f>BDP(A41&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C41">
-        <f>BDP(A41,"CRNCY")</f>
+        <f>BDP(A41&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D41">
-        <f>BDP(A41,"CNTRY_OF_RISK")</f>
+        <f>BDP(A41&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E41">
-        <f>BDP(A41,"CPN")/100</f>
+        <f>BDP(A41&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F41">
-        <f>BDP(A41,"CPN_FREQ")</f>
+        <f>BDP(A41&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G41">
-        <f>BDP(A41,"DAY_CNT_DES")</f>
+        <f>BDP(A41&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H41">
-        <f>BDP(A41,"MATURITY")</f>
+        <f>BDP(A41&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I41">
-        <f>BDP(A41,"FIRST_CPN_DT")</f>
+        <f>BDP(A41&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42">
-        <f>BDP(A42,"SECURITY_DES")</f>
+        <f>BDP(A42&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C42">
-        <f>BDP(A42,"CRNCY")</f>
+        <f>BDP(A42&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D42">
-        <f>BDP(A42,"CNTRY_OF_RISK")</f>
+        <f>BDP(A42&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E42">
-        <f>BDP(A42,"CPN")/100</f>
+        <f>BDP(A42&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F42">
-        <f>BDP(A42,"CPN_FREQ")</f>
+        <f>BDP(A42&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G42">
-        <f>BDP(A42,"DAY_CNT_DES")</f>
+        <f>BDP(A42&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H42">
-        <f>BDP(A42,"MATURITY")</f>
+        <f>BDP(A42&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I42">
-        <f>BDP(A42,"FIRST_CPN_DT")</f>
+        <f>BDP(A42&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43">
-        <f>BDP(A43,"SECURITY_DES")</f>
+        <f>BDP(A43&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C43">
-        <f>BDP(A43,"CRNCY")</f>
+        <f>BDP(A43&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D43">
-        <f>BDP(A43,"CNTRY_OF_RISK")</f>
+        <f>BDP(A43&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E43">
-        <f>BDP(A43,"CPN")/100</f>
+        <f>BDP(A43&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F43">
-        <f>BDP(A43,"CPN_FREQ")</f>
+        <f>BDP(A43&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G43">
-        <f>BDP(A43,"DAY_CNT_DES")</f>
+        <f>BDP(A43&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H43">
-        <f>BDP(A43,"MATURITY")</f>
+        <f>BDP(A43&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I43">
-        <f>BDP(A43,"FIRST_CPN_DT")</f>
+        <f>BDP(A43&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44">
-        <f>BDP(A44,"SECURITY_DES")</f>
+        <f>BDP(A44&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C44">
-        <f>BDP(A44,"CRNCY")</f>
+        <f>BDP(A44&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D44">
-        <f>BDP(A44,"CNTRY_OF_RISK")</f>
+        <f>BDP(A44&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E44">
-        <f>BDP(A44,"CPN")/100</f>
+        <f>BDP(A44&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F44">
-        <f>BDP(A44,"CPN_FREQ")</f>
+        <f>BDP(A44&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G44">
-        <f>BDP(A44,"DAY_CNT_DES")</f>
+        <f>BDP(A44&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H44">
-        <f>BDP(A44,"MATURITY")</f>
+        <f>BDP(A44&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I44">
-        <f>BDP(A44,"FIRST_CPN_DT")</f>
+        <f>BDP(A44&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45">
-        <f>BDP(A45,"SECURITY_DES")</f>
+        <f>BDP(A45&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C45">
-        <f>BDP(A45,"CRNCY")</f>
+        <f>BDP(A45&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D45">
-        <f>BDP(A45,"CNTRY_OF_RISK")</f>
+        <f>BDP(A45&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E45">
-        <f>BDP(A45,"CPN")/100</f>
+        <f>BDP(A45&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F45">
-        <f>BDP(A45,"CPN_FREQ")</f>
+        <f>BDP(A45&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G45">
-        <f>BDP(A45,"DAY_CNT_DES")</f>
+        <f>BDP(A45&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H45">
-        <f>BDP(A45,"MATURITY")</f>
+        <f>BDP(A45&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I45">
-        <f>BDP(A45,"FIRST_CPN_DT")</f>
+        <f>BDP(A45&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="B46">
-        <f>BDP(A46,"SECURITY_DES")</f>
+        <f>BDP(A46&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C46">
-        <f>BDP(A46,"CRNCY")</f>
+        <f>BDP(A46&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D46">
-        <f>BDP(A46,"CNTRY_OF_RISK")</f>
+        <f>BDP(A46&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E46">
-        <f>BDP(A46,"CPN")/100</f>
+        <f>BDP(A46&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F46">
-        <f>BDP(A46,"CPN_FREQ")</f>
+        <f>BDP(A46&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G46">
-        <f>BDP(A46,"DAY_CNT_DES")</f>
+        <f>BDP(A46&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H46">
-        <f>BDP(A46,"MATURITY")</f>
+        <f>BDP(A46&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I46">
-        <f>BDP(A46,"FIRST_CPN_DT")</f>
+        <f>BDP(A46&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47">
-        <f>BDP(A47,"SECURITY_DES")</f>
+        <f>BDP(A47&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C47">
-        <f>BDP(A47,"CRNCY")</f>
+        <f>BDP(A47&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D47">
-        <f>BDP(A47,"CNTRY_OF_RISK")</f>
+        <f>BDP(A47&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E47">
-        <f>BDP(A47,"CPN")/100</f>
+        <f>BDP(A47&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F47">
-        <f>BDP(A47,"CPN_FREQ")</f>
+        <f>BDP(A47&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G47">
-        <f>BDP(A47,"DAY_CNT_DES")</f>
+        <f>BDP(A47&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H47">
-        <f>BDP(A47,"MATURITY")</f>
+        <f>BDP(A47&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I47">
-        <f>BDP(A47,"FIRST_CPN_DT")</f>
+        <f>BDP(A47&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="B48">
-        <f>BDP(A48,"SECURITY_DES")</f>
+        <f>BDP(A48&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C48">
-        <f>BDP(A48,"CRNCY")</f>
+        <f>BDP(A48&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D48">
-        <f>BDP(A48,"CNTRY_OF_RISK")</f>
+        <f>BDP(A48&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E48">
-        <f>BDP(A48,"CPN")/100</f>
+        <f>BDP(A48&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F48">
-        <f>BDP(A48,"CPN_FREQ")</f>
+        <f>BDP(A48&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G48">
-        <f>BDP(A48,"DAY_CNT_DES")</f>
+        <f>BDP(A48&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H48">
-        <f>BDP(A48,"MATURITY")</f>
+        <f>BDP(A48&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I48">
-        <f>BDP(A48,"FIRST_CPN_DT")</f>
+        <f>BDP(A48&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="B49">
-        <f>BDP(A49,"SECURITY_DES")</f>
+        <f>BDP(A49&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C49">
-        <f>BDP(A49,"CRNCY")</f>
+        <f>BDP(A49&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D49">
-        <f>BDP(A49,"CNTRY_OF_RISK")</f>
+        <f>BDP(A49&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E49">
-        <f>BDP(A49,"CPN")/100</f>
+        <f>BDP(A49&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F49">
-        <f>BDP(A49,"CPN_FREQ")</f>
+        <f>BDP(A49&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G49">
-        <f>BDP(A49,"DAY_CNT_DES")</f>
+        <f>BDP(A49&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H49">
-        <f>BDP(A49,"MATURITY")</f>
+        <f>BDP(A49&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I49">
-        <f>BDP(A49,"FIRST_CPN_DT")</f>
+        <f>BDP(A49&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="B50">
-        <f>BDP(A50,"SECURITY_DES")</f>
+        <f>BDP(A50&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C50">
-        <f>BDP(A50,"CRNCY")</f>
+        <f>BDP(A50&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D50">
-        <f>BDP(A50,"CNTRY_OF_RISK")</f>
+        <f>BDP(A50&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E50">
-        <f>BDP(A50,"CPN")/100</f>
+        <f>BDP(A50&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F50">
-        <f>BDP(A50,"CPN_FREQ")</f>
+        <f>BDP(A50&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G50">
-        <f>BDP(A50,"DAY_CNT_DES")</f>
+        <f>BDP(A50&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H50">
-        <f>BDP(A50,"MATURITY")</f>
+        <f>BDP(A50&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I50">
-        <f>BDP(A50,"FIRST_CPN_DT")</f>
+        <f>BDP(A50&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="B51">
-        <f>BDP(A51,"SECURITY_DES")</f>
+        <f>BDP(A51&amp;" Corp","SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C51">
-        <f>BDP(A51,"CRNCY")</f>
+        <f>BDP(A51&amp;" Corp","CRNCY")</f>
         <v/>
       </c>
       <c r="D51">
-        <f>BDP(A51,"CNTRY_OF_RISK")</f>
+        <f>BDP(A51&amp;" Corp","CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E51">
-        <f>BDP(A51,"CPN")/100</f>
+        <f>BDP(A51&amp;" Corp","CPN")/100</f>
         <v/>
       </c>
       <c r="F51">
-        <f>BDP(A51,"CPN_FREQ")</f>
+        <f>BDP(A51&amp;" Corp","CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G51">
-        <f>BDP(A51,"DAY_CNT_DES")</f>
+        <f>BDP(A51&amp;" Corp","DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H51">
-        <f>BDP(A51,"MATURITY")</f>
+        <f>BDP(A51&amp;" Corp","MATURITY")</f>
         <v/>
       </c>
       <c r="I51">
-        <f>BDP(A51,"FIRST_CPN_DT")</f>
+        <f>BDP(A51&amp;" Corp","FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
@@ -2946,29 +2951,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BBG Ticker</t>
+          <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Start (YYYYMMDD)</t>
+          <t>PX_LAST</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>End (YYYYMMDD)</t>
+          <t>End</t>
         </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <f>BDH(A1,"PX_LAST",B1,C1,"Fill","0","Dates","1")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Redesign History sheet to horizontal column-pair layout with @BDH formulas
Replaces the old vertical 510-row-block layout (YYYYMMDD integers, one
block per CUSIP-range stacked down A/B/C) with a horizontal column-pair
layout: one column pair per CUSIP (A/B, C/D, E/F, ...), dates in
mm/dd/yyyy, shared end-date in A2 (today-1), shared field label in B2.

Formula per bond i: =@BDH({col}1,B2,{start_ref},A2,"fill=p","days=a")
  - Bond 0 start date in B1; bonds 1+ start dates in D2, F2, F2, ...
  - Multiple gap ranges for the same CUSIP are collapsed to min(start)
    since find_price_gaps already returns only missing ranges

read_history_from_template reads column-pairs from row 4 downward,
keyed by the ordered_cusips list saved in backfill_state.json.

_fetch_bdh_via_excel (xlwings auto path) updated to use mm/dd/yyyy
dates and =@BDH syntax for consistency.

https://claude.ai/code/session_018koFNQ47GjPqFMqjAKyQE4
</commit_message>
<xml_diff>
--- a/projects/02-pnl-dashboard/templates/bloomberg_prices.xlsx
+++ b/projects/02-pnl-dashboard/templates/bloomberg_prices.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Live MTM" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Static" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="History" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,10 +33,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,13 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +435,7 @@
   <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -449,7 +444,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CUSIP</t>
+          <t>BBG Ticker</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -470,701 +465,701 @@
     </row>
     <row r="2">
       <c r="B2">
-        <f>BDP(A2&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A2,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C2">
-        <f>BDP(A2&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A2,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>BDP(A2&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A2,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="B3">
-        <f>BDP(A3&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A3,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C3">
-        <f>BDP(A3&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A3,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>BDP(A3&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A3,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="B4">
-        <f>BDP(A4&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A4,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C4">
-        <f>BDP(A4&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A4,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>BDP(A4&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A4,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="B5">
-        <f>BDP(A5&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A5,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C5">
-        <f>BDP(A5&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A5,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>BDP(A5&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A5,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6">
-        <f>BDP(A6&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A6,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>BDP(A6&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A6,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>BDP(A6&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A6,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7">
-        <f>BDP(A7&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A7,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C7">
-        <f>BDP(A7&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A7,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D7">
-        <f>BDP(A7&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A7,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8">
-        <f>BDP(A8&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A8,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C8">
-        <f>BDP(A8&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A8,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D8">
-        <f>BDP(A8&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A8,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9">
-        <f>BDP(A9&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A9,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C9">
-        <f>BDP(A9&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A9,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D9">
-        <f>BDP(A9&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A9,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10">
-        <f>BDP(A10&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A10,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C10">
-        <f>BDP(A10&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A10,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D10">
-        <f>BDP(A10&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A10,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="B11">
-        <f>BDP(A11&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A11,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>BDP(A11&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A11,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D11">
-        <f>BDP(A11&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A11,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="B12">
-        <f>BDP(A12&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A12,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>BDP(A12&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A12,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>BDP(A12&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A12,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13">
-        <f>BDP(A13&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A13,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>BDP(A13&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A13,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D13">
-        <f>BDP(A13&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A13,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14">
-        <f>BDP(A14&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A14,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>BDP(A14&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A14,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D14">
-        <f>BDP(A14&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A14,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="B15">
-        <f>BDP(A15&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A15,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>BDP(A15&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A15,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D15">
-        <f>BDP(A15&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A15,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16">
-        <f>BDP(A16&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A16,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>BDP(A16&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A16,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D16">
-        <f>BDP(A16&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A16,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17">
-        <f>BDP(A17&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A17,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>BDP(A17&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A17,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D17">
-        <f>BDP(A17&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A17,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18">
-        <f>BDP(A18&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A18,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>BDP(A18&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A18,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D18">
-        <f>BDP(A18&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A18,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19">
-        <f>BDP(A19&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A19,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>BDP(A19&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A19,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D19">
-        <f>BDP(A19&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A19,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20">
-        <f>BDP(A20&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A20,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>BDP(A20&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A20,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D20">
-        <f>BDP(A20&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A20,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21">
-        <f>BDP(A21&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A21,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>BDP(A21&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A21,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D21">
-        <f>BDP(A21&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A21,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="B22">
-        <f>BDP(A22&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A22,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>BDP(A22&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A22,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D22">
-        <f>BDP(A22&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A22,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="B23">
-        <f>BDP(A23&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A23,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>BDP(A23&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A23,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>BDP(A23&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A23,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24">
-        <f>BDP(A24&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A24,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>BDP(A24&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A24,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>BDP(A24&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A24,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25">
-        <f>BDP(A25&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A25,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>BDP(A25&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A25,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>BDP(A25&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A25,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26">
-        <f>BDP(A26&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A26,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>BDP(A26&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A26,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D26">
-        <f>BDP(A26&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A26,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27">
-        <f>BDP(A27&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A27,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>BDP(A27&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A27,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>BDP(A27&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A27,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28">
-        <f>BDP(A28&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A28,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>BDP(A28&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A28,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D28">
-        <f>BDP(A28&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A28,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29">
-        <f>BDP(A29&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A29,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>BDP(A29&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A29,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D29">
-        <f>BDP(A29&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A29,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30">
-        <f>BDP(A30&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A30,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>BDP(A30&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A30,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D30">
-        <f>BDP(A30&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A30,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="B31">
-        <f>BDP(A31&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A31,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>BDP(A31&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A31,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D31">
-        <f>BDP(A31&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A31,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32">
-        <f>BDP(A32&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A32,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>BDP(A32&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A32,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D32">
-        <f>BDP(A32&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A32,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33">
-        <f>BDP(A33&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A33,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C33">
-        <f>BDP(A33&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A33,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>BDP(A33&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A33,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34">
-        <f>BDP(A34&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A34,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C34">
-        <f>BDP(A34&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A34,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>BDP(A34&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A34,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35">
-        <f>BDP(A35&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A35,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C35">
-        <f>BDP(A35&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A35,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D35">
-        <f>BDP(A35&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A35,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36">
-        <f>BDP(A36&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A36,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C36">
-        <f>BDP(A36&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A36,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D36">
-        <f>BDP(A36&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A36,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37">
-        <f>BDP(A37&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A37,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C37">
-        <f>BDP(A37&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A37,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D37">
-        <f>BDP(A37&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A37,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="B38">
-        <f>BDP(A38&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A38,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C38">
-        <f>BDP(A38&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A38,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D38">
-        <f>BDP(A38&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A38,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39">
-        <f>BDP(A39&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A39,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C39">
-        <f>BDP(A39&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A39,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D39">
-        <f>BDP(A39&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A39,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="B40">
-        <f>BDP(A40&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A40,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C40">
-        <f>BDP(A40&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A40,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D40">
-        <f>BDP(A40&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A40,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="B41">
-        <f>BDP(A41&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A41,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C41">
-        <f>BDP(A41&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A41,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D41">
-        <f>BDP(A41&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A41,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42">
-        <f>BDP(A42&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A42,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C42">
-        <f>BDP(A42&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A42,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D42">
-        <f>BDP(A42&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A42,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43">
-        <f>BDP(A43&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A43,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C43">
-        <f>BDP(A43&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A43,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D43">
-        <f>BDP(A43&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A43,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44">
-        <f>BDP(A44&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A44,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C44">
-        <f>BDP(A44&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A44,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D44">
-        <f>BDP(A44&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A44,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45">
-        <f>BDP(A45&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A45,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C45">
-        <f>BDP(A45&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A45,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D45">
-        <f>BDP(A45&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A45,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="B46">
-        <f>BDP(A46&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A46,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C46">
-        <f>BDP(A46&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A46,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D46">
-        <f>BDP(A46&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A46,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47">
-        <f>BDP(A47&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A47,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C47">
-        <f>BDP(A47&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A47,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D47">
-        <f>BDP(A47&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A47,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="B48">
-        <f>BDP(A48&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A48,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C48">
-        <f>BDP(A48&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A48,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D48">
-        <f>BDP(A48&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A48,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="B49">
-        <f>BDP(A49&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A49,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C49">
-        <f>BDP(A49&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A49,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D49">
-        <f>BDP(A49&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A49,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="B50">
-        <f>BDP(A50&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A50,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C50">
-        <f>BDP(A50&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A50,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D50">
-        <f>BDP(A50&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A50,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="B51">
-        <f>BDP(A51&amp;" Corp","PX_LAST")</f>
+        <f>BDP(A51,"PX_LAST")</f>
         <v/>
       </c>
       <c r="C51">
-        <f>BDP(A51&amp;" Corp","YAS_ASW_SPREAD")</f>
+        <f>BDP(A51,"YAS_ASW_SPREAD")</f>
         <v/>
       </c>
       <c r="D51">
-        <f>BDP(A51&amp;" Corp","YLD_YTM_MID")</f>
+        <f>BDP(A51,"YLD_YTM_MID")</f>
         <v/>
       </c>
     </row>
@@ -1182,7 +1177,7 @@
   <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -1196,7 +1191,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>cusip</t>
+          <t>bbg_ticker</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1242,1701 +1237,1701 @@
     </row>
     <row r="2">
       <c r="B2">
-        <f>BDP(A2&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A2,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C2">
-        <f>BDP(A2&amp;" Corp","CRNCY")</f>
+        <f>BDP(A2,"CRNCY")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>BDP(A2&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A2,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E2">
-        <f>BDP(A2&amp;" Corp","CPN")/100</f>
+        <f>BDP(A2,"CPN")/100</f>
         <v/>
       </c>
       <c r="F2">
-        <f>BDP(A2&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A2,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G2">
-        <f>BDP(A2&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A2,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H2">
-        <f>BDP(A2&amp;" Corp","MATURITY")</f>
+        <f>BDP(A2,"MATURITY")</f>
         <v/>
       </c>
       <c r="I2">
-        <f>BDP(A2&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A2,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="B3">
-        <f>BDP(A3&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A3,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C3">
-        <f>BDP(A3&amp;" Corp","CRNCY")</f>
+        <f>BDP(A3,"CRNCY")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>BDP(A3&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A3,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E3">
-        <f>BDP(A3&amp;" Corp","CPN")/100</f>
+        <f>BDP(A3,"CPN")/100</f>
         <v/>
       </c>
       <c r="F3">
-        <f>BDP(A3&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A3,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G3">
-        <f>BDP(A3&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A3,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H3">
-        <f>BDP(A3&amp;" Corp","MATURITY")</f>
+        <f>BDP(A3,"MATURITY")</f>
         <v/>
       </c>
       <c r="I3">
-        <f>BDP(A3&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A3,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="B4">
-        <f>BDP(A4&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A4,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C4">
-        <f>BDP(A4&amp;" Corp","CRNCY")</f>
+        <f>BDP(A4,"CRNCY")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>BDP(A4&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A4,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E4">
-        <f>BDP(A4&amp;" Corp","CPN")/100</f>
+        <f>BDP(A4,"CPN")/100</f>
         <v/>
       </c>
       <c r="F4">
-        <f>BDP(A4&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A4,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G4">
-        <f>BDP(A4&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A4,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H4">
-        <f>BDP(A4&amp;" Corp","MATURITY")</f>
+        <f>BDP(A4,"MATURITY")</f>
         <v/>
       </c>
       <c r="I4">
-        <f>BDP(A4&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A4,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="B5">
-        <f>BDP(A5&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A5,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C5">
-        <f>BDP(A5&amp;" Corp","CRNCY")</f>
+        <f>BDP(A5,"CRNCY")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>BDP(A5&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A5,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E5">
-        <f>BDP(A5&amp;" Corp","CPN")/100</f>
+        <f>BDP(A5,"CPN")/100</f>
         <v/>
       </c>
       <c r="F5">
-        <f>BDP(A5&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A5,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G5">
-        <f>BDP(A5&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A5,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H5">
-        <f>BDP(A5&amp;" Corp","MATURITY")</f>
+        <f>BDP(A5,"MATURITY")</f>
         <v/>
       </c>
       <c r="I5">
-        <f>BDP(A5&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A5,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6">
-        <f>BDP(A6&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A6,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>BDP(A6&amp;" Corp","CRNCY")</f>
+        <f>BDP(A6,"CRNCY")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>BDP(A6&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A6,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E6">
-        <f>BDP(A6&amp;" Corp","CPN")/100</f>
+        <f>BDP(A6,"CPN")/100</f>
         <v/>
       </c>
       <c r="F6">
-        <f>BDP(A6&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A6,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G6">
-        <f>BDP(A6&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A6,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H6">
-        <f>BDP(A6&amp;" Corp","MATURITY")</f>
+        <f>BDP(A6,"MATURITY")</f>
         <v/>
       </c>
       <c r="I6">
-        <f>BDP(A6&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A6,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7">
-        <f>BDP(A7&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A7,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C7">
-        <f>BDP(A7&amp;" Corp","CRNCY")</f>
+        <f>BDP(A7,"CRNCY")</f>
         <v/>
       </c>
       <c r="D7">
-        <f>BDP(A7&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A7,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E7">
-        <f>BDP(A7&amp;" Corp","CPN")/100</f>
+        <f>BDP(A7,"CPN")/100</f>
         <v/>
       </c>
       <c r="F7">
-        <f>BDP(A7&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A7,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G7">
-        <f>BDP(A7&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A7,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H7">
-        <f>BDP(A7&amp;" Corp","MATURITY")</f>
+        <f>BDP(A7,"MATURITY")</f>
         <v/>
       </c>
       <c r="I7">
-        <f>BDP(A7&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A7,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8">
-        <f>BDP(A8&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A8,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C8">
-        <f>BDP(A8&amp;" Corp","CRNCY")</f>
+        <f>BDP(A8,"CRNCY")</f>
         <v/>
       </c>
       <c r="D8">
-        <f>BDP(A8&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A8,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E8">
-        <f>BDP(A8&amp;" Corp","CPN")/100</f>
+        <f>BDP(A8,"CPN")/100</f>
         <v/>
       </c>
       <c r="F8">
-        <f>BDP(A8&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A8,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G8">
-        <f>BDP(A8&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A8,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H8">
-        <f>BDP(A8&amp;" Corp","MATURITY")</f>
+        <f>BDP(A8,"MATURITY")</f>
         <v/>
       </c>
       <c r="I8">
-        <f>BDP(A8&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A8,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9">
-        <f>BDP(A9&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A9,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C9">
-        <f>BDP(A9&amp;" Corp","CRNCY")</f>
+        <f>BDP(A9,"CRNCY")</f>
         <v/>
       </c>
       <c r="D9">
-        <f>BDP(A9&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A9,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E9">
-        <f>BDP(A9&amp;" Corp","CPN")/100</f>
+        <f>BDP(A9,"CPN")/100</f>
         <v/>
       </c>
       <c r="F9">
-        <f>BDP(A9&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A9,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G9">
-        <f>BDP(A9&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A9,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H9">
-        <f>BDP(A9&amp;" Corp","MATURITY")</f>
+        <f>BDP(A9,"MATURITY")</f>
         <v/>
       </c>
       <c r="I9">
-        <f>BDP(A9&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A9,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10">
-        <f>BDP(A10&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A10,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C10">
-        <f>BDP(A10&amp;" Corp","CRNCY")</f>
+        <f>BDP(A10,"CRNCY")</f>
         <v/>
       </c>
       <c r="D10">
-        <f>BDP(A10&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A10,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E10">
-        <f>BDP(A10&amp;" Corp","CPN")/100</f>
+        <f>BDP(A10,"CPN")/100</f>
         <v/>
       </c>
       <c r="F10">
-        <f>BDP(A10&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A10,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G10">
-        <f>BDP(A10&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A10,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H10">
-        <f>BDP(A10&amp;" Corp","MATURITY")</f>
+        <f>BDP(A10,"MATURITY")</f>
         <v/>
       </c>
       <c r="I10">
-        <f>BDP(A10&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A10,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="B11">
-        <f>BDP(A11&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A11,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>BDP(A11&amp;" Corp","CRNCY")</f>
+        <f>BDP(A11,"CRNCY")</f>
         <v/>
       </c>
       <c r="D11">
-        <f>BDP(A11&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A11,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E11">
-        <f>BDP(A11&amp;" Corp","CPN")/100</f>
+        <f>BDP(A11,"CPN")/100</f>
         <v/>
       </c>
       <c r="F11">
-        <f>BDP(A11&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A11,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G11">
-        <f>BDP(A11&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A11,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H11">
-        <f>BDP(A11&amp;" Corp","MATURITY")</f>
+        <f>BDP(A11,"MATURITY")</f>
         <v/>
       </c>
       <c r="I11">
-        <f>BDP(A11&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A11,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="B12">
-        <f>BDP(A12&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A12,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>BDP(A12&amp;" Corp","CRNCY")</f>
+        <f>BDP(A12,"CRNCY")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>BDP(A12&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A12,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E12">
-        <f>BDP(A12&amp;" Corp","CPN")/100</f>
+        <f>BDP(A12,"CPN")/100</f>
         <v/>
       </c>
       <c r="F12">
-        <f>BDP(A12&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A12,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G12">
-        <f>BDP(A12&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A12,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H12">
-        <f>BDP(A12&amp;" Corp","MATURITY")</f>
+        <f>BDP(A12,"MATURITY")</f>
         <v/>
       </c>
       <c r="I12">
-        <f>BDP(A12&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A12,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13">
-        <f>BDP(A13&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A13,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>BDP(A13&amp;" Corp","CRNCY")</f>
+        <f>BDP(A13,"CRNCY")</f>
         <v/>
       </c>
       <c r="D13">
-        <f>BDP(A13&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A13,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E13">
-        <f>BDP(A13&amp;" Corp","CPN")/100</f>
+        <f>BDP(A13,"CPN")/100</f>
         <v/>
       </c>
       <c r="F13">
-        <f>BDP(A13&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A13,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G13">
-        <f>BDP(A13&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A13,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H13">
-        <f>BDP(A13&amp;" Corp","MATURITY")</f>
+        <f>BDP(A13,"MATURITY")</f>
         <v/>
       </c>
       <c r="I13">
-        <f>BDP(A13&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A13,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14">
-        <f>BDP(A14&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A14,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>BDP(A14&amp;" Corp","CRNCY")</f>
+        <f>BDP(A14,"CRNCY")</f>
         <v/>
       </c>
       <c r="D14">
-        <f>BDP(A14&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A14,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E14">
-        <f>BDP(A14&amp;" Corp","CPN")/100</f>
+        <f>BDP(A14,"CPN")/100</f>
         <v/>
       </c>
       <c r="F14">
-        <f>BDP(A14&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A14,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G14">
-        <f>BDP(A14&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A14,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H14">
-        <f>BDP(A14&amp;" Corp","MATURITY")</f>
+        <f>BDP(A14,"MATURITY")</f>
         <v/>
       </c>
       <c r="I14">
-        <f>BDP(A14&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A14,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="B15">
-        <f>BDP(A15&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A15,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>BDP(A15&amp;" Corp","CRNCY")</f>
+        <f>BDP(A15,"CRNCY")</f>
         <v/>
       </c>
       <c r="D15">
-        <f>BDP(A15&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A15,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E15">
-        <f>BDP(A15&amp;" Corp","CPN")/100</f>
+        <f>BDP(A15,"CPN")/100</f>
         <v/>
       </c>
       <c r="F15">
-        <f>BDP(A15&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A15,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G15">
-        <f>BDP(A15&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A15,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H15">
-        <f>BDP(A15&amp;" Corp","MATURITY")</f>
+        <f>BDP(A15,"MATURITY")</f>
         <v/>
       </c>
       <c r="I15">
-        <f>BDP(A15&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A15,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16">
-        <f>BDP(A16&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A16,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>BDP(A16&amp;" Corp","CRNCY")</f>
+        <f>BDP(A16,"CRNCY")</f>
         <v/>
       </c>
       <c r="D16">
-        <f>BDP(A16&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A16,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E16">
-        <f>BDP(A16&amp;" Corp","CPN")/100</f>
+        <f>BDP(A16,"CPN")/100</f>
         <v/>
       </c>
       <c r="F16">
-        <f>BDP(A16&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A16,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G16">
-        <f>BDP(A16&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A16,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H16">
-        <f>BDP(A16&amp;" Corp","MATURITY")</f>
+        <f>BDP(A16,"MATURITY")</f>
         <v/>
       </c>
       <c r="I16">
-        <f>BDP(A16&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A16,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17">
-        <f>BDP(A17&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A17,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>BDP(A17&amp;" Corp","CRNCY")</f>
+        <f>BDP(A17,"CRNCY")</f>
         <v/>
       </c>
       <c r="D17">
-        <f>BDP(A17&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A17,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E17">
-        <f>BDP(A17&amp;" Corp","CPN")/100</f>
+        <f>BDP(A17,"CPN")/100</f>
         <v/>
       </c>
       <c r="F17">
-        <f>BDP(A17&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A17,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G17">
-        <f>BDP(A17&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A17,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H17">
-        <f>BDP(A17&amp;" Corp","MATURITY")</f>
+        <f>BDP(A17,"MATURITY")</f>
         <v/>
       </c>
       <c r="I17">
-        <f>BDP(A17&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A17,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18">
-        <f>BDP(A18&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A18,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>BDP(A18&amp;" Corp","CRNCY")</f>
+        <f>BDP(A18,"CRNCY")</f>
         <v/>
       </c>
       <c r="D18">
-        <f>BDP(A18&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A18,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E18">
-        <f>BDP(A18&amp;" Corp","CPN")/100</f>
+        <f>BDP(A18,"CPN")/100</f>
         <v/>
       </c>
       <c r="F18">
-        <f>BDP(A18&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A18,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G18">
-        <f>BDP(A18&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A18,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H18">
-        <f>BDP(A18&amp;" Corp","MATURITY")</f>
+        <f>BDP(A18,"MATURITY")</f>
         <v/>
       </c>
       <c r="I18">
-        <f>BDP(A18&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A18,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19">
-        <f>BDP(A19&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A19,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>BDP(A19&amp;" Corp","CRNCY")</f>
+        <f>BDP(A19,"CRNCY")</f>
         <v/>
       </c>
       <c r="D19">
-        <f>BDP(A19&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A19,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E19">
-        <f>BDP(A19&amp;" Corp","CPN")/100</f>
+        <f>BDP(A19,"CPN")/100</f>
         <v/>
       </c>
       <c r="F19">
-        <f>BDP(A19&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A19,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G19">
-        <f>BDP(A19&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A19,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H19">
-        <f>BDP(A19&amp;" Corp","MATURITY")</f>
+        <f>BDP(A19,"MATURITY")</f>
         <v/>
       </c>
       <c r="I19">
-        <f>BDP(A19&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A19,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20">
-        <f>BDP(A20&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A20,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>BDP(A20&amp;" Corp","CRNCY")</f>
+        <f>BDP(A20,"CRNCY")</f>
         <v/>
       </c>
       <c r="D20">
-        <f>BDP(A20&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A20,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E20">
-        <f>BDP(A20&amp;" Corp","CPN")/100</f>
+        <f>BDP(A20,"CPN")/100</f>
         <v/>
       </c>
       <c r="F20">
-        <f>BDP(A20&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A20,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G20">
-        <f>BDP(A20&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A20,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H20">
-        <f>BDP(A20&amp;" Corp","MATURITY")</f>
+        <f>BDP(A20,"MATURITY")</f>
         <v/>
       </c>
       <c r="I20">
-        <f>BDP(A20&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A20,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21">
-        <f>BDP(A21&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A21,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>BDP(A21&amp;" Corp","CRNCY")</f>
+        <f>BDP(A21,"CRNCY")</f>
         <v/>
       </c>
       <c r="D21">
-        <f>BDP(A21&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A21,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E21">
-        <f>BDP(A21&amp;" Corp","CPN")/100</f>
+        <f>BDP(A21,"CPN")/100</f>
         <v/>
       </c>
       <c r="F21">
-        <f>BDP(A21&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A21,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G21">
-        <f>BDP(A21&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A21,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H21">
-        <f>BDP(A21&amp;" Corp","MATURITY")</f>
+        <f>BDP(A21,"MATURITY")</f>
         <v/>
       </c>
       <c r="I21">
-        <f>BDP(A21&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A21,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="B22">
-        <f>BDP(A22&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A22,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>BDP(A22&amp;" Corp","CRNCY")</f>
+        <f>BDP(A22,"CRNCY")</f>
         <v/>
       </c>
       <c r="D22">
-        <f>BDP(A22&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A22,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E22">
-        <f>BDP(A22&amp;" Corp","CPN")/100</f>
+        <f>BDP(A22,"CPN")/100</f>
         <v/>
       </c>
       <c r="F22">
-        <f>BDP(A22&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A22,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G22">
-        <f>BDP(A22&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A22,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H22">
-        <f>BDP(A22&amp;" Corp","MATURITY")</f>
+        <f>BDP(A22,"MATURITY")</f>
         <v/>
       </c>
       <c r="I22">
-        <f>BDP(A22&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A22,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="B23">
-        <f>BDP(A23&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A23,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>BDP(A23&amp;" Corp","CRNCY")</f>
+        <f>BDP(A23,"CRNCY")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>BDP(A23&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A23,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E23">
-        <f>BDP(A23&amp;" Corp","CPN")/100</f>
+        <f>BDP(A23,"CPN")/100</f>
         <v/>
       </c>
       <c r="F23">
-        <f>BDP(A23&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A23,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G23">
-        <f>BDP(A23&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A23,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H23">
-        <f>BDP(A23&amp;" Corp","MATURITY")</f>
+        <f>BDP(A23,"MATURITY")</f>
         <v/>
       </c>
       <c r="I23">
-        <f>BDP(A23&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A23,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24">
-        <f>BDP(A24&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A24,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>BDP(A24&amp;" Corp","CRNCY")</f>
+        <f>BDP(A24,"CRNCY")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>BDP(A24&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A24,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E24">
-        <f>BDP(A24&amp;" Corp","CPN")/100</f>
+        <f>BDP(A24,"CPN")/100</f>
         <v/>
       </c>
       <c r="F24">
-        <f>BDP(A24&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A24,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G24">
-        <f>BDP(A24&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A24,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H24">
-        <f>BDP(A24&amp;" Corp","MATURITY")</f>
+        <f>BDP(A24,"MATURITY")</f>
         <v/>
       </c>
       <c r="I24">
-        <f>BDP(A24&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A24,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25">
-        <f>BDP(A25&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A25,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>BDP(A25&amp;" Corp","CRNCY")</f>
+        <f>BDP(A25,"CRNCY")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>BDP(A25&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A25,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E25">
-        <f>BDP(A25&amp;" Corp","CPN")/100</f>
+        <f>BDP(A25,"CPN")/100</f>
         <v/>
       </c>
       <c r="F25">
-        <f>BDP(A25&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A25,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G25">
-        <f>BDP(A25&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A25,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H25">
-        <f>BDP(A25&amp;" Corp","MATURITY")</f>
+        <f>BDP(A25,"MATURITY")</f>
         <v/>
       </c>
       <c r="I25">
-        <f>BDP(A25&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A25,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26">
-        <f>BDP(A26&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A26,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>BDP(A26&amp;" Corp","CRNCY")</f>
+        <f>BDP(A26,"CRNCY")</f>
         <v/>
       </c>
       <c r="D26">
-        <f>BDP(A26&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A26,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E26">
-        <f>BDP(A26&amp;" Corp","CPN")/100</f>
+        <f>BDP(A26,"CPN")/100</f>
         <v/>
       </c>
       <c r="F26">
-        <f>BDP(A26&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A26,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G26">
-        <f>BDP(A26&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A26,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H26">
-        <f>BDP(A26&amp;" Corp","MATURITY")</f>
+        <f>BDP(A26,"MATURITY")</f>
         <v/>
       </c>
       <c r="I26">
-        <f>BDP(A26&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A26,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27">
-        <f>BDP(A27&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A27,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>BDP(A27&amp;" Corp","CRNCY")</f>
+        <f>BDP(A27,"CRNCY")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>BDP(A27&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A27,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E27">
-        <f>BDP(A27&amp;" Corp","CPN")/100</f>
+        <f>BDP(A27,"CPN")/100</f>
         <v/>
       </c>
       <c r="F27">
-        <f>BDP(A27&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A27,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G27">
-        <f>BDP(A27&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A27,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H27">
-        <f>BDP(A27&amp;" Corp","MATURITY")</f>
+        <f>BDP(A27,"MATURITY")</f>
         <v/>
       </c>
       <c r="I27">
-        <f>BDP(A27&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A27,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28">
-        <f>BDP(A28&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A28,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>BDP(A28&amp;" Corp","CRNCY")</f>
+        <f>BDP(A28,"CRNCY")</f>
         <v/>
       </c>
       <c r="D28">
-        <f>BDP(A28&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A28,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E28">
-        <f>BDP(A28&amp;" Corp","CPN")/100</f>
+        <f>BDP(A28,"CPN")/100</f>
         <v/>
       </c>
       <c r="F28">
-        <f>BDP(A28&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A28,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G28">
-        <f>BDP(A28&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A28,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H28">
-        <f>BDP(A28&amp;" Corp","MATURITY")</f>
+        <f>BDP(A28,"MATURITY")</f>
         <v/>
       </c>
       <c r="I28">
-        <f>BDP(A28&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A28,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29">
-        <f>BDP(A29&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A29,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>BDP(A29&amp;" Corp","CRNCY")</f>
+        <f>BDP(A29,"CRNCY")</f>
         <v/>
       </c>
       <c r="D29">
-        <f>BDP(A29&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A29,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E29">
-        <f>BDP(A29&amp;" Corp","CPN")/100</f>
+        <f>BDP(A29,"CPN")/100</f>
         <v/>
       </c>
       <c r="F29">
-        <f>BDP(A29&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A29,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G29">
-        <f>BDP(A29&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A29,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H29">
-        <f>BDP(A29&amp;" Corp","MATURITY")</f>
+        <f>BDP(A29,"MATURITY")</f>
         <v/>
       </c>
       <c r="I29">
-        <f>BDP(A29&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A29,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30">
-        <f>BDP(A30&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A30,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>BDP(A30&amp;" Corp","CRNCY")</f>
+        <f>BDP(A30,"CRNCY")</f>
         <v/>
       </c>
       <c r="D30">
-        <f>BDP(A30&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A30,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E30">
-        <f>BDP(A30&amp;" Corp","CPN")/100</f>
+        <f>BDP(A30,"CPN")/100</f>
         <v/>
       </c>
       <c r="F30">
-        <f>BDP(A30&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A30,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G30">
-        <f>BDP(A30&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A30,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H30">
-        <f>BDP(A30&amp;" Corp","MATURITY")</f>
+        <f>BDP(A30,"MATURITY")</f>
         <v/>
       </c>
       <c r="I30">
-        <f>BDP(A30&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A30,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="B31">
-        <f>BDP(A31&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A31,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>BDP(A31&amp;" Corp","CRNCY")</f>
+        <f>BDP(A31,"CRNCY")</f>
         <v/>
       </c>
       <c r="D31">
-        <f>BDP(A31&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A31,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E31">
-        <f>BDP(A31&amp;" Corp","CPN")/100</f>
+        <f>BDP(A31,"CPN")/100</f>
         <v/>
       </c>
       <c r="F31">
-        <f>BDP(A31&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A31,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G31">
-        <f>BDP(A31&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A31,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H31">
-        <f>BDP(A31&amp;" Corp","MATURITY")</f>
+        <f>BDP(A31,"MATURITY")</f>
         <v/>
       </c>
       <c r="I31">
-        <f>BDP(A31&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A31,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32">
-        <f>BDP(A32&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A32,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>BDP(A32&amp;" Corp","CRNCY")</f>
+        <f>BDP(A32,"CRNCY")</f>
         <v/>
       </c>
       <c r="D32">
-        <f>BDP(A32&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A32,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E32">
-        <f>BDP(A32&amp;" Corp","CPN")/100</f>
+        <f>BDP(A32,"CPN")/100</f>
         <v/>
       </c>
       <c r="F32">
-        <f>BDP(A32&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A32,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G32">
-        <f>BDP(A32&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A32,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H32">
-        <f>BDP(A32&amp;" Corp","MATURITY")</f>
+        <f>BDP(A32,"MATURITY")</f>
         <v/>
       </c>
       <c r="I32">
-        <f>BDP(A32&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A32,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33">
-        <f>BDP(A33&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A33,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C33">
-        <f>BDP(A33&amp;" Corp","CRNCY")</f>
+        <f>BDP(A33,"CRNCY")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>BDP(A33&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A33,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E33">
-        <f>BDP(A33&amp;" Corp","CPN")/100</f>
+        <f>BDP(A33,"CPN")/100</f>
         <v/>
       </c>
       <c r="F33">
-        <f>BDP(A33&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A33,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G33">
-        <f>BDP(A33&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A33,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H33">
-        <f>BDP(A33&amp;" Corp","MATURITY")</f>
+        <f>BDP(A33,"MATURITY")</f>
         <v/>
       </c>
       <c r="I33">
-        <f>BDP(A33&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A33,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34">
-        <f>BDP(A34&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A34,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C34">
-        <f>BDP(A34&amp;" Corp","CRNCY")</f>
+        <f>BDP(A34,"CRNCY")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>BDP(A34&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A34,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E34">
-        <f>BDP(A34&amp;" Corp","CPN")/100</f>
+        <f>BDP(A34,"CPN")/100</f>
         <v/>
       </c>
       <c r="F34">
-        <f>BDP(A34&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A34,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G34">
-        <f>BDP(A34&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A34,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H34">
-        <f>BDP(A34&amp;" Corp","MATURITY")</f>
+        <f>BDP(A34,"MATURITY")</f>
         <v/>
       </c>
       <c r="I34">
-        <f>BDP(A34&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A34,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35">
-        <f>BDP(A35&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A35,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C35">
-        <f>BDP(A35&amp;" Corp","CRNCY")</f>
+        <f>BDP(A35,"CRNCY")</f>
         <v/>
       </c>
       <c r="D35">
-        <f>BDP(A35&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A35,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E35">
-        <f>BDP(A35&amp;" Corp","CPN")/100</f>
+        <f>BDP(A35,"CPN")/100</f>
         <v/>
       </c>
       <c r="F35">
-        <f>BDP(A35&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A35,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G35">
-        <f>BDP(A35&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A35,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H35">
-        <f>BDP(A35&amp;" Corp","MATURITY")</f>
+        <f>BDP(A35,"MATURITY")</f>
         <v/>
       </c>
       <c r="I35">
-        <f>BDP(A35&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A35,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36">
-        <f>BDP(A36&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A36,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C36">
-        <f>BDP(A36&amp;" Corp","CRNCY")</f>
+        <f>BDP(A36,"CRNCY")</f>
         <v/>
       </c>
       <c r="D36">
-        <f>BDP(A36&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A36,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E36">
-        <f>BDP(A36&amp;" Corp","CPN")/100</f>
+        <f>BDP(A36,"CPN")/100</f>
         <v/>
       </c>
       <c r="F36">
-        <f>BDP(A36&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A36,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G36">
-        <f>BDP(A36&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A36,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H36">
-        <f>BDP(A36&amp;" Corp","MATURITY")</f>
+        <f>BDP(A36,"MATURITY")</f>
         <v/>
       </c>
       <c r="I36">
-        <f>BDP(A36&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A36,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37">
-        <f>BDP(A37&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A37,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C37">
-        <f>BDP(A37&amp;" Corp","CRNCY")</f>
+        <f>BDP(A37,"CRNCY")</f>
         <v/>
       </c>
       <c r="D37">
-        <f>BDP(A37&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A37,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E37">
-        <f>BDP(A37&amp;" Corp","CPN")/100</f>
+        <f>BDP(A37,"CPN")/100</f>
         <v/>
       </c>
       <c r="F37">
-        <f>BDP(A37&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A37,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G37">
-        <f>BDP(A37&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A37,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H37">
-        <f>BDP(A37&amp;" Corp","MATURITY")</f>
+        <f>BDP(A37,"MATURITY")</f>
         <v/>
       </c>
       <c r="I37">
-        <f>BDP(A37&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A37,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="B38">
-        <f>BDP(A38&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A38,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C38">
-        <f>BDP(A38&amp;" Corp","CRNCY")</f>
+        <f>BDP(A38,"CRNCY")</f>
         <v/>
       </c>
       <c r="D38">
-        <f>BDP(A38&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A38,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E38">
-        <f>BDP(A38&amp;" Corp","CPN")/100</f>
+        <f>BDP(A38,"CPN")/100</f>
         <v/>
       </c>
       <c r="F38">
-        <f>BDP(A38&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A38,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G38">
-        <f>BDP(A38&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A38,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H38">
-        <f>BDP(A38&amp;" Corp","MATURITY")</f>
+        <f>BDP(A38,"MATURITY")</f>
         <v/>
       </c>
       <c r="I38">
-        <f>BDP(A38&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A38,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39">
-        <f>BDP(A39&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A39,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C39">
-        <f>BDP(A39&amp;" Corp","CRNCY")</f>
+        <f>BDP(A39,"CRNCY")</f>
         <v/>
       </c>
       <c r="D39">
-        <f>BDP(A39&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A39,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E39">
-        <f>BDP(A39&amp;" Corp","CPN")/100</f>
+        <f>BDP(A39,"CPN")/100</f>
         <v/>
       </c>
       <c r="F39">
-        <f>BDP(A39&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A39,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G39">
-        <f>BDP(A39&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A39,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H39">
-        <f>BDP(A39&amp;" Corp","MATURITY")</f>
+        <f>BDP(A39,"MATURITY")</f>
         <v/>
       </c>
       <c r="I39">
-        <f>BDP(A39&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A39,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="B40">
-        <f>BDP(A40&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A40,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C40">
-        <f>BDP(A40&amp;" Corp","CRNCY")</f>
+        <f>BDP(A40,"CRNCY")</f>
         <v/>
       </c>
       <c r="D40">
-        <f>BDP(A40&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A40,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E40">
-        <f>BDP(A40&amp;" Corp","CPN")/100</f>
+        <f>BDP(A40,"CPN")/100</f>
         <v/>
       </c>
       <c r="F40">
-        <f>BDP(A40&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A40,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G40">
-        <f>BDP(A40&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A40,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H40">
-        <f>BDP(A40&amp;" Corp","MATURITY")</f>
+        <f>BDP(A40,"MATURITY")</f>
         <v/>
       </c>
       <c r="I40">
-        <f>BDP(A40&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A40,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="B41">
-        <f>BDP(A41&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A41,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C41">
-        <f>BDP(A41&amp;" Corp","CRNCY")</f>
+        <f>BDP(A41,"CRNCY")</f>
         <v/>
       </c>
       <c r="D41">
-        <f>BDP(A41&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A41,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E41">
-        <f>BDP(A41&amp;" Corp","CPN")/100</f>
+        <f>BDP(A41,"CPN")/100</f>
         <v/>
       </c>
       <c r="F41">
-        <f>BDP(A41&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A41,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G41">
-        <f>BDP(A41&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A41,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H41">
-        <f>BDP(A41&amp;" Corp","MATURITY")</f>
+        <f>BDP(A41,"MATURITY")</f>
         <v/>
       </c>
       <c r="I41">
-        <f>BDP(A41&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A41,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42">
-        <f>BDP(A42&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A42,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C42">
-        <f>BDP(A42&amp;" Corp","CRNCY")</f>
+        <f>BDP(A42,"CRNCY")</f>
         <v/>
       </c>
       <c r="D42">
-        <f>BDP(A42&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A42,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E42">
-        <f>BDP(A42&amp;" Corp","CPN")/100</f>
+        <f>BDP(A42,"CPN")/100</f>
         <v/>
       </c>
       <c r="F42">
-        <f>BDP(A42&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A42,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G42">
-        <f>BDP(A42&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A42,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H42">
-        <f>BDP(A42&amp;" Corp","MATURITY")</f>
+        <f>BDP(A42,"MATURITY")</f>
         <v/>
       </c>
       <c r="I42">
-        <f>BDP(A42&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A42,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43">
-        <f>BDP(A43&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A43,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C43">
-        <f>BDP(A43&amp;" Corp","CRNCY")</f>
+        <f>BDP(A43,"CRNCY")</f>
         <v/>
       </c>
       <c r="D43">
-        <f>BDP(A43&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A43,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E43">
-        <f>BDP(A43&amp;" Corp","CPN")/100</f>
+        <f>BDP(A43,"CPN")/100</f>
         <v/>
       </c>
       <c r="F43">
-        <f>BDP(A43&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A43,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G43">
-        <f>BDP(A43&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A43,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H43">
-        <f>BDP(A43&amp;" Corp","MATURITY")</f>
+        <f>BDP(A43,"MATURITY")</f>
         <v/>
       </c>
       <c r="I43">
-        <f>BDP(A43&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A43,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44">
-        <f>BDP(A44&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A44,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C44">
-        <f>BDP(A44&amp;" Corp","CRNCY")</f>
+        <f>BDP(A44,"CRNCY")</f>
         <v/>
       </c>
       <c r="D44">
-        <f>BDP(A44&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A44,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E44">
-        <f>BDP(A44&amp;" Corp","CPN")/100</f>
+        <f>BDP(A44,"CPN")/100</f>
         <v/>
       </c>
       <c r="F44">
-        <f>BDP(A44&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A44,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G44">
-        <f>BDP(A44&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A44,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H44">
-        <f>BDP(A44&amp;" Corp","MATURITY")</f>
+        <f>BDP(A44,"MATURITY")</f>
         <v/>
       </c>
       <c r="I44">
-        <f>BDP(A44&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A44,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45">
-        <f>BDP(A45&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A45,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C45">
-        <f>BDP(A45&amp;" Corp","CRNCY")</f>
+        <f>BDP(A45,"CRNCY")</f>
         <v/>
       </c>
       <c r="D45">
-        <f>BDP(A45&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A45,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E45">
-        <f>BDP(A45&amp;" Corp","CPN")/100</f>
+        <f>BDP(A45,"CPN")/100</f>
         <v/>
       </c>
       <c r="F45">
-        <f>BDP(A45&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A45,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G45">
-        <f>BDP(A45&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A45,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H45">
-        <f>BDP(A45&amp;" Corp","MATURITY")</f>
+        <f>BDP(A45,"MATURITY")</f>
         <v/>
       </c>
       <c r="I45">
-        <f>BDP(A45&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A45,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="B46">
-        <f>BDP(A46&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A46,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C46">
-        <f>BDP(A46&amp;" Corp","CRNCY")</f>
+        <f>BDP(A46,"CRNCY")</f>
         <v/>
       </c>
       <c r="D46">
-        <f>BDP(A46&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A46,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E46">
-        <f>BDP(A46&amp;" Corp","CPN")/100</f>
+        <f>BDP(A46,"CPN")/100</f>
         <v/>
       </c>
       <c r="F46">
-        <f>BDP(A46&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A46,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G46">
-        <f>BDP(A46&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A46,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H46">
-        <f>BDP(A46&amp;" Corp","MATURITY")</f>
+        <f>BDP(A46,"MATURITY")</f>
         <v/>
       </c>
       <c r="I46">
-        <f>BDP(A46&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A46,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47">
-        <f>BDP(A47&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A47,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C47">
-        <f>BDP(A47&amp;" Corp","CRNCY")</f>
+        <f>BDP(A47,"CRNCY")</f>
         <v/>
       </c>
       <c r="D47">
-        <f>BDP(A47&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A47,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E47">
-        <f>BDP(A47&amp;" Corp","CPN")/100</f>
+        <f>BDP(A47,"CPN")/100</f>
         <v/>
       </c>
       <c r="F47">
-        <f>BDP(A47&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A47,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G47">
-        <f>BDP(A47&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A47,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H47">
-        <f>BDP(A47&amp;" Corp","MATURITY")</f>
+        <f>BDP(A47,"MATURITY")</f>
         <v/>
       </c>
       <c r="I47">
-        <f>BDP(A47&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A47,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="B48">
-        <f>BDP(A48&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A48,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C48">
-        <f>BDP(A48&amp;" Corp","CRNCY")</f>
+        <f>BDP(A48,"CRNCY")</f>
         <v/>
       </c>
       <c r="D48">
-        <f>BDP(A48&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A48,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E48">
-        <f>BDP(A48&amp;" Corp","CPN")/100</f>
+        <f>BDP(A48,"CPN")/100</f>
         <v/>
       </c>
       <c r="F48">
-        <f>BDP(A48&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A48,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G48">
-        <f>BDP(A48&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A48,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H48">
-        <f>BDP(A48&amp;" Corp","MATURITY")</f>
+        <f>BDP(A48,"MATURITY")</f>
         <v/>
       </c>
       <c r="I48">
-        <f>BDP(A48&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A48,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="B49">
-        <f>BDP(A49&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A49,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C49">
-        <f>BDP(A49&amp;" Corp","CRNCY")</f>
+        <f>BDP(A49,"CRNCY")</f>
         <v/>
       </c>
       <c r="D49">
-        <f>BDP(A49&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A49,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E49">
-        <f>BDP(A49&amp;" Corp","CPN")/100</f>
+        <f>BDP(A49,"CPN")/100</f>
         <v/>
       </c>
       <c r="F49">
-        <f>BDP(A49&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A49,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G49">
-        <f>BDP(A49&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A49,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H49">
-        <f>BDP(A49&amp;" Corp","MATURITY")</f>
+        <f>BDP(A49,"MATURITY")</f>
         <v/>
       </c>
       <c r="I49">
-        <f>BDP(A49&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A49,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="B50">
-        <f>BDP(A50&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A50,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C50">
-        <f>BDP(A50&amp;" Corp","CRNCY")</f>
+        <f>BDP(A50,"CRNCY")</f>
         <v/>
       </c>
       <c r="D50">
-        <f>BDP(A50&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A50,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E50">
-        <f>BDP(A50&amp;" Corp","CPN")/100</f>
+        <f>BDP(A50,"CPN")/100</f>
         <v/>
       </c>
       <c r="F50">
-        <f>BDP(A50&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A50,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G50">
-        <f>BDP(A50&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A50,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H50">
-        <f>BDP(A50&amp;" Corp","MATURITY")</f>
+        <f>BDP(A50,"MATURITY")</f>
         <v/>
       </c>
       <c r="I50">
-        <f>BDP(A50&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A50,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="B51">
-        <f>BDP(A51&amp;" Corp","SECURITY_DES")</f>
+        <f>BDP(A51,"SECURITY_DES")</f>
         <v/>
       </c>
       <c r="C51">
-        <f>BDP(A51&amp;" Corp","CRNCY")</f>
+        <f>BDP(A51,"CRNCY")</f>
         <v/>
       </c>
       <c r="D51">
-        <f>BDP(A51&amp;" Corp","CNTRY_OF_RISK")</f>
+        <f>BDP(A51,"CNTRY_OF_RISK")</f>
         <v/>
       </c>
       <c r="E51">
-        <f>BDP(A51&amp;" Corp","CPN")/100</f>
+        <f>BDP(A51,"CPN")/100</f>
         <v/>
       </c>
       <c r="F51">
-        <f>BDP(A51&amp;" Corp","CPN_FREQ")</f>
+        <f>BDP(A51,"CPN_FREQ")</f>
         <v/>
       </c>
       <c r="G51">
-        <f>BDP(A51&amp;" Corp","DAY_CNT_DES")</f>
+        <f>BDP(A51,"DAY_CNT_DES")</f>
         <v/>
       </c>
       <c r="H51">
-        <f>BDP(A51&amp;" Corp","MATURITY")</f>
+        <f>BDP(A51,"MATURITY")</f>
         <v/>
       </c>
       <c r="I51">
-        <f>BDP(A51&amp;" Corp","FIRST_CPN_DT")</f>
+        <f>BDP(A51,"FIRST_CPN_DT")</f>
         <v/>
       </c>
     </row>
@@ -2951,34 +2946,86 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>25714PFB9 Corp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>04/30/2025</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>195325ER2 Corp</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>25714PEF1 Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>06/03/2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>PX_LAST</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
-          <t>End</t>
+          <t>05/20/2025</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>05/12/2025</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
-        <f>BDH(A1,"PX_LAST",B1,C1,"Fill","0","Dates","1")</f>
+      <c r="A3">
+        <f>@BDH(A1,B2,B1,A2,"fill=p","days=a")</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>@BDH(C1,B2,D2,A2,"fill=p","days=a")</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>@BDH(E1,B2,F2,A2,"fill=p","days=a")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(pnl-dashboard): robust Static sheet reader; handle #N/A maturity_date
- read_static_from_template() no longer hardcodes range(1,10). Headers are
  now read dynamically until the first empty cell, so the reader works
  correctly regardless of how many columns the template has (past or future).
- maturity_date field now treats None/#N/A explicitly: if Bloomberg returns
  #N/A for MATURITY (bond matured or wrong ticker), the row is skipped with
  a clear warning instead of being imported with a null maturity that then
  triggers the "missing required field" warning on every dashboard load.
- Regenerated templates/bloomberg_prices.xlsx to ensure the committed file
  matches the current create_bloomberg_template.py (maturity_date present at
  col 8, first_coupon_date at col 9).

https://claude.ai/code/session_018koFNQ47GjPqFMqjAKyQE4
</commit_message>
<xml_diff>
--- a/projects/02-pnl-dashboard/templates/bloomberg_prices.xlsx
+++ b/projects/02-pnl-dashboard/templates/bloomberg_prices.xlsx
@@ -2946,7 +2946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2974,59 +2974,20 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>25714PFB9 Corp</t>
+          <t>BBG Ticker</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>04/30/2025</t>
+          <t>End Date (mm/dd/yyyy)</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>195325ER2 Corp</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>25714PEF1 Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>06/03/2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>PX_LAST</t>
         </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>05/20/2025</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>05/12/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <f>@BDH(A1,B2,B1,A2,"fill=p","days=a")</f>
-        <v/>
-      </c>
-      <c r="C3">
-        <f>@BDH(C1,B2,D2,A2,"fill=p","days=a")</f>
-        <v/>
-      </c>
-      <c r="E3">
-        <f>@BDH(E1,B2,F2,A2,"fill=p","days=a")</f>
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>